<commit_message>
Documenta la fusión del PR #22: defecto 26 corregido, CP-079 y CP-080 y límite de reservas
Registro de Defectos con los 26 corregidos. Planilla con 80 casos (77 aprobados). Escenario 4 de FS-HU-14 en la planilla de historias y nota en el Product Backlog. DAS 1.22 sin referencias a revisión pendiente. Guía 2.4 y control actualizados (diagrama UML de componentes implementado).
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/Plantilla_Historias_Usuario_con_instructivo.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/Plantilla_Historias_Usuario_con_instructivo.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:J94"/>
+  <dimension ref="A1:K93"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
     <col width="1.44140625" customWidth="1" style="5" min="1" max="1"/>
@@ -1861,10 +1861,10 @@
       </c>
     </row>
     <row r="48" ht="55" customHeight="1">
-      <c r="B48" s="20" t="n"/>
-      <c r="C48" s="20" t="n"/>
-      <c r="D48" s="20" t="n"/>
-      <c r="E48" s="20" t="n"/>
+      <c r="B48" s="22" t="n"/>
+      <c r="C48" s="22" t="n"/>
+      <c r="D48" s="22" t="n"/>
+      <c r="E48" s="22" t="n"/>
       <c r="F48" s="8" t="n">
         <v>3</v>
       </c>
@@ -1889,1169 +1889,1198 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="55" customHeight="1"/>
-    <row r="50" ht="55" customHeight="1">
-      <c r="B50" s="6" t="inlineStr">
+    <row r="49" ht="55" customHeight="1">
+      <c r="B49" s="22" t="n"/>
+      <c r="C49" s="22" t="n"/>
+      <c r="D49" s="22" t="n"/>
+      <c r="E49" s="22" t="n"/>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>Límite de una reserva activa por profesional</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>En caso que el usuario ya tiene una reserva pendiente o confirmada para un horario futuro con ese profesional</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>cuando intenta reservar otra hora con el mismo profesional</t>
+        </is>
+      </c>
+      <c r="J49" s="6" t="inlineStr">
+        <is>
+          <t>el sistema no crea la reserva, se lo avisa antes de escribir el mensaje y le indica que primero cancele la reserva activa en "Mis citas"; las citas que ya pasaron no cuentan para este límite (decisión del Product Owner del 12-10-2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="55" customHeight="1"/>
+    <row r="51" ht="55" customHeight="1">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>FS-HU-15</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>Necesito recuperar mi contraseña mediante un enlace enviado a mi correo</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de volver a acceder a mi cuenta si la olvido</t>
         </is>
       </c>
-      <c r="F50" s="8" t="n">
+      <c r="F51" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G50" s="6" t="inlineStr">
+      <c r="G51" s="6" t="inlineStr">
         <is>
           <t>Solicitar enlace de recuperación</t>
         </is>
       </c>
-      <c r="H50" s="6" t="inlineStr">
+      <c r="H51" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario olvidó su contraseña</t>
         </is>
       </c>
-      <c r="I50" s="6" t="inlineStr">
+      <c r="I51" s="6" t="inlineStr">
         <is>
           <t>cuando escribe su correo en "¿Olvidaste tu contraseña?" y presiona "Enviar enlace"</t>
         </is>
       </c>
-      <c r="J50" s="6" t="inlineStr">
+      <c r="J51" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra siempre el mismo mensaje de confirmación y, si el correo está registrado, envía un correo con un enlace válido por 60 minutos</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="55" customHeight="1">
-      <c r="B51" s="22" t="n"/>
-      <c r="C51" s="22" t="n"/>
-      <c r="D51" s="22" t="n"/>
-      <c r="E51" s="22" t="n"/>
-      <c r="F51" s="8" t="n">
+    <row r="52" ht="55" customHeight="1">
+      <c r="B52" s="22" t="n"/>
+      <c r="C52" s="22" t="n"/>
+      <c r="D52" s="22" t="n"/>
+      <c r="E52" s="22" t="n"/>
+      <c r="F52" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G51" s="6" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>Restablecer la contraseña</t>
         </is>
       </c>
-      <c r="H51" s="6" t="inlineStr">
+      <c r="H52" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario abre un enlace de recuperación vigente</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr">
+      <c r="I52" s="6" t="inlineStr">
         <is>
           <t>cuando escribe una contraseña nueva de al menos 8 caracteres y su confirmación coincide</t>
         </is>
       </c>
-      <c r="J51" s="6" t="inlineStr">
+      <c r="J52" s="6" t="inlineStr">
         <is>
           <t>el sistema actualiza la contraseña, inutiliza el enlace y permite iniciar sesión con la contraseña nueva</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="55" customHeight="1">
-      <c r="B52" s="20" t="n"/>
-      <c r="C52" s="20" t="n"/>
-      <c r="D52" s="20" t="n"/>
-      <c r="E52" s="20" t="n"/>
-      <c r="F52" s="8" t="n">
+    <row r="53" ht="55" customHeight="1">
+      <c r="B53" s="20" t="n"/>
+      <c r="C53" s="20" t="n"/>
+      <c r="D53" s="20" t="n"/>
+      <c r="E53" s="20" t="n"/>
+      <c r="F53" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G52" s="6" t="inlineStr">
+      <c r="G53" s="6" t="inlineStr">
         <is>
           <t>Enlace vencido o usado</t>
         </is>
       </c>
-      <c r="H52" s="6" t="inlineStr">
+      <c r="H53" s="6" t="inlineStr">
         <is>
           <t>En caso que el enlace ya venció, ya se usó o fue alterado</t>
         </is>
       </c>
-      <c r="I52" s="6" t="inlineStr">
+      <c r="I53" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario intenta restablecer la contraseña</t>
         </is>
       </c>
-      <c r="J52" s="6" t="inlineStr">
+      <c r="J53" s="6" t="inlineStr">
         <is>
           <t>el sistema no cambia la contraseña e indica que debe solicitar un enlace nuevo</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="55" customHeight="1"/>
-    <row r="54" ht="55" customHeight="1">
-      <c r="B54" s="6" t="inlineStr">
+    <row r="54" ht="55" customHeight="1"/>
+    <row r="55" ht="55" customHeight="1">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>FS-HU-16</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>Como un usuario o profesional</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>Necesito registrarme e iniciar sesión con mi cuenta de Google</t>
         </is>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de acceder sin crear ni recordar otra contraseña</t>
         </is>
       </c>
-      <c r="F54" s="8" t="n">
+      <c r="F55" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G54" s="6" t="inlineStr">
+      <c r="G55" s="6" t="inlineStr">
         <is>
           <t>Primer acceso con Google</t>
         </is>
       </c>
-      <c r="H54" s="6" t="inlineStr">
+      <c r="H55" s="6" t="inlineStr">
         <is>
           <t>En caso que la persona no tiene cuenta en FitSearch</t>
         </is>
       </c>
-      <c r="I54" s="6" t="inlineStr">
+      <c r="I55" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Continuar con Google" y autoriza el acceso</t>
         </is>
       </c>
-      <c r="J54" s="6" t="inlineStr">
+      <c r="J55" s="6" t="inlineStr">
         <is>
           <t>el sistema crea la cuenta y su perfil vacío, deja la sesión iniciada y le pide elegir su tipo de cuenta en el primer paso del perfil</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="55" customHeight="1">
-      <c r="B55" s="22" t="n"/>
-      <c r="C55" s="22" t="n"/>
-      <c r="D55" s="22" t="n"/>
-      <c r="E55" s="22" t="n"/>
-      <c r="F55" s="8" t="n">
+    <row r="56" ht="55" customHeight="1">
+      <c r="B56" s="22" t="n"/>
+      <c r="C56" s="22" t="n"/>
+      <c r="D56" s="22" t="n"/>
+      <c r="E56" s="22" t="n"/>
+      <c r="F56" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G55" s="6" t="inlineStr">
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>Cuenta existente con el mismo correo</t>
         </is>
       </c>
-      <c r="H55" s="6" t="inlineStr">
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>En caso que ya existe una cuenta registrada con el correo de Google</t>
         </is>
       </c>
-      <c r="I55" s="6" t="inlineStr">
+      <c r="I56" s="6" t="inlineStr">
         <is>
           <t>cuando la persona continúa con Google</t>
         </is>
       </c>
-      <c r="J55" s="6" t="inlineStr">
+      <c r="J56" s="6" t="inlineStr">
         <is>
           <t>el sistema vincula la cuenta de Google a la cuenta existente e inicia la sesión sin crear un usuario duplicado</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="55" customHeight="1">
-      <c r="B56" s="20" t="n"/>
-      <c r="C56" s="20" t="n"/>
-      <c r="D56" s="20" t="n"/>
-      <c r="E56" s="20" t="n"/>
-      <c r="F56" s="8" t="n">
+    <row r="57" ht="55" customHeight="1">
+      <c r="B57" s="20" t="n"/>
+      <c r="C57" s="20" t="n"/>
+      <c r="D57" s="20" t="n"/>
+      <c r="E57" s="20" t="n"/>
+      <c r="F57" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G56" s="6" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>Acceso con Google inválido</t>
         </is>
       </c>
-      <c r="H56" s="6" t="inlineStr">
+      <c r="H57" s="6" t="inlineStr">
         <is>
           <t>En caso que la validación de Google falla o el correo no está verificado</t>
         </is>
       </c>
-      <c r="I56" s="6" t="inlineStr">
+      <c r="I57" s="6" t="inlineStr">
         <is>
           <t>cuando el sistema recibe la solicitud de acceso</t>
         </is>
       </c>
-      <c r="J56" s="6" t="inlineStr">
+      <c r="J57" s="6" t="inlineStr">
         <is>
           <t>el sistema rechaza el acceso y muestra un mensaje de error sin crear la cuenta</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="55" customHeight="1"/>
-    <row r="58" ht="55" customHeight="1">
-      <c r="B58" s="6" t="inlineStr">
+    <row r="58" ht="55" customHeight="1"/>
+    <row r="59" ht="55" customHeight="1">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>FS-HU-17</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>Como un usuario o profesional</t>
         </is>
       </c>
-      <c r="D58" s="6" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>Necesito confirmar mi contraseña al registrarme y decidir si mantener mi sesión iniciada</t>
         </is>
       </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de acceder a las funciones que me corresponden de forma cómoda y segura</t>
         </is>
       </c>
-      <c r="F58" s="8" t="n">
+      <c r="F59" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G58" s="6" t="inlineStr">
+      <c r="G59" s="6" t="inlineStr">
         <is>
           <t>Registro sin elegir rol</t>
         </is>
       </c>
-      <c r="H58" s="6" t="inlineStr">
+      <c r="H59" s="6" t="inlineStr">
         <is>
           <t>En caso que la persona completa el formulario de registro</t>
         </is>
       </c>
-      <c r="I58" s="6" t="inlineStr">
+      <c r="I59" s="6" t="inlineStr">
         <is>
           <t>cuando confirma el registro</t>
         </is>
       </c>
-      <c r="J58" s="6" t="inlineStr">
+      <c r="J59" s="6" t="inlineStr">
         <is>
           <t>el sistema crea la cuenta como usuario y le pide elegir su tipo de cuenta en el perfil; nunca permite registrarse como administrador</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="55" customHeight="1">
-      <c r="B59" s="22" t="n"/>
-      <c r="C59" s="22" t="n"/>
-      <c r="D59" s="22" t="n"/>
-      <c r="E59" s="22" t="n"/>
-      <c r="F59" s="8" t="n">
+    <row r="60" ht="55" customHeight="1">
+      <c r="B60" s="22" t="n"/>
+      <c r="C60" s="22" t="n"/>
+      <c r="D60" s="22" t="n"/>
+      <c r="E60" s="22" t="n"/>
+      <c r="F60" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G59" s="6" t="inlineStr">
+      <c r="G60" s="6" t="inlineStr">
         <is>
           <t>Contraseñas distintas</t>
         </is>
       </c>
-      <c r="H59" s="6" t="inlineStr">
+      <c r="H60" s="6" t="inlineStr">
         <is>
           <t>En caso que la contraseña y su confirmación no coinciden</t>
         </is>
       </c>
-      <c r="I59" s="6" t="inlineStr">
+      <c r="I60" s="6" t="inlineStr">
         <is>
           <t>cuando la persona intenta registrarse</t>
         </is>
       </c>
-      <c r="J59" s="6" t="inlineStr">
+      <c r="J60" s="6" t="inlineStr">
         <is>
           <t>el sistema no crea la cuenta e indica que las contraseñas no coinciden</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="55" customHeight="1">
-      <c r="B60" s="20" t="n"/>
-      <c r="C60" s="20" t="n"/>
-      <c r="D60" s="20" t="n"/>
-      <c r="E60" s="20" t="n"/>
-      <c r="F60" s="8" t="n">
+    <row r="61" ht="55" customHeight="1">
+      <c r="B61" s="20" t="n"/>
+      <c r="C61" s="20" t="n"/>
+      <c r="D61" s="20" t="n"/>
+      <c r="E61" s="20" t="n"/>
+      <c r="F61" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G60" s="6" t="inlineStr">
+      <c r="G61" s="6" t="inlineStr">
         <is>
           <t>Recordarme</t>
         </is>
       </c>
-      <c r="H60" s="6" t="inlineStr">
+      <c r="H61" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario inicia sesión</t>
         </is>
       </c>
-      <c r="I60" s="6" t="inlineStr">
+      <c r="I61" s="6" t="inlineStr">
         <is>
           <t>cuando marca o no marca "Recordarme"</t>
         </is>
       </c>
-      <c r="J60" s="6" t="inlineStr">
+      <c r="J61" s="6" t="inlineStr">
         <is>
           <t>si lo marcó, la sesión se mantiene hasta 30 días aunque cierre el navegador; si no, la sesión termina al cerrar el navegador</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="55" customHeight="1"/>
-    <row r="62" ht="55" customHeight="1">
-      <c r="B62" s="6" t="inlineStr">
+    <row r="62" ht="55" customHeight="1"/>
+    <row r="63" ht="55" customHeight="1">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>FS-HU-18</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr">
+      <c r="C63" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D62" s="6" t="inlineStr">
+      <c r="D63" s="6" t="inlineStr">
         <is>
           <t>Necesito indicar mi objetivo principal y mi estilo de vida (comidas al día y horas de sueño)</t>
         </is>
       </c>
-      <c r="E62" s="6" t="inlineStr">
+      <c r="E63" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de recibir una orientación acorde a lo que busco lograr</t>
         </is>
       </c>
-      <c r="F62" s="8" t="n">
+      <c r="F63" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G62" s="6" t="inlineStr">
+      <c r="G63" s="6" t="inlineStr">
         <is>
           <t>Guardar objetivos y estilo de vida</t>
         </is>
       </c>
-      <c r="H62" s="6" t="inlineStr">
+      <c r="H63" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario completó sus datos personales en el asistente</t>
         </is>
       </c>
-      <c r="I62" s="6" t="inlineStr">
+      <c r="I63" s="6" t="inlineStr">
         <is>
           <t>cuando elige su objetivo principal, las comidas al día y las horas de sueño y presiona "Siguiente"</t>
         </is>
       </c>
-      <c r="J62" s="6" t="inlineStr">
+      <c r="J63" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda la información y avanza al paso de información de salud</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="55" customHeight="1">
-      <c r="B63" s="22" t="n"/>
-      <c r="C63" s="22" t="n"/>
-      <c r="D63" s="22" t="n"/>
-      <c r="E63" s="22" t="n"/>
-      <c r="F63" s="8" t="n">
+    <row r="64" ht="55" customHeight="1">
+      <c r="B64" s="22" t="n"/>
+      <c r="C64" s="22" t="n"/>
+      <c r="D64" s="22" t="n"/>
+      <c r="E64" s="22" t="n"/>
+      <c r="F64" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G63" s="6" t="inlineStr">
+      <c r="G64" s="6" t="inlineStr">
         <is>
           <t>Datos incompletos</t>
         </is>
       </c>
-      <c r="H63" s="6" t="inlineStr">
+      <c r="H64" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario no responde alguna de las preguntas</t>
         </is>
       </c>
-      <c r="I63" s="6" t="inlineStr">
+      <c r="I64" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Siguiente"</t>
         </is>
       </c>
-      <c r="J63" s="6" t="inlineStr">
+      <c r="J64" s="6" t="inlineStr">
         <is>
           <t>el sistema no guarda y señala cada pregunta pendiente</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="55" customHeight="1">
-      <c r="B64" s="20" t="n"/>
-      <c r="C64" s="20" t="n"/>
-      <c r="D64" s="20" t="n"/>
-      <c r="E64" s="20" t="n"/>
-      <c r="F64" s="8" t="n">
+    <row r="65" ht="55" customHeight="1">
+      <c r="B65" s="20" t="n"/>
+      <c r="C65" s="20" t="n"/>
+      <c r="D65" s="20" t="n"/>
+      <c r="E65" s="20" t="n"/>
+      <c r="F65" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G64" s="6" t="inlineStr">
+      <c r="G65" s="6" t="inlineStr">
         <is>
           <t>Editar desde el resumen</t>
         </is>
       </c>
-      <c r="H64" s="6" t="inlineStr">
+      <c r="H65" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ya completó su perfil</t>
         </is>
       </c>
-      <c r="I64" s="6" t="inlineStr">
+      <c r="I65" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Editar" en Objetivos y estilo de vida, cambia su objetivo y guarda</t>
         </is>
       </c>
-      <c r="J64" s="6" t="inlineStr">
+      <c r="J65" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda el cambio y vuelve al resumen mostrando el objetivo actualizado</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="55" customHeight="1"/>
-    <row r="66" ht="55" customHeight="1">
-      <c r="B66" s="6" t="inlineStr">
+    <row r="66" ht="55" customHeight="1"/>
+    <row r="67" ht="55" customHeight="1">
+      <c r="B67" s="6" t="inlineStr">
         <is>
           <t>FS-HU-19</t>
         </is>
       </c>
-      <c r="C66" s="6" t="inlineStr">
+      <c r="C67" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D66" s="6" t="inlineStr">
+      <c r="D67" s="6" t="inlineStr">
         <is>
           <t>Necesito registrar mis condiciones médicas, medicamentos y alergias de forma confidencial</t>
         </is>
       </c>
-      <c r="E66" s="6" t="inlineStr">
+      <c r="E67" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de recibir recomendaciones más seguras y adecuadas a mi situación</t>
         </is>
       </c>
-      <c r="F66" s="8" t="n">
+      <c r="F67" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G66" s="6" t="inlineStr">
+      <c r="G67" s="6" t="inlineStr">
         <is>
           <t>Guardar información de salud</t>
         </is>
       </c>
-      <c r="H66" s="6" t="inlineStr">
+      <c r="H67" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario está en el paso de información de salud</t>
         </is>
       </c>
-      <c r="I66" s="6" t="inlineStr">
+      <c r="I67" s="6" t="inlineStr">
         <is>
           <t>cuando marca sus condiciones médicas, indica si toma medicamentos (y de qué tipo) y sus alergias, y presiona "Siguiente"</t>
         </is>
       </c>
-      <c r="J66" s="6" t="inlineStr">
+      <c r="J67" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda la información, muestra "¡Información guardada!" con el requerimiento calórico estimado y luego el resumen del perfil</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="55" customHeight="1">
-      <c r="B67" s="22" t="n"/>
-      <c r="C67" s="22" t="n"/>
-      <c r="D67" s="22" t="n"/>
-      <c r="E67" s="22" t="n"/>
-      <c r="F67" s="8" t="n">
+    <row r="68" ht="55" customHeight="1">
+      <c r="B68" s="22" t="n"/>
+      <c r="C68" s="22" t="n"/>
+      <c r="D68" s="22" t="n"/>
+      <c r="E68" s="22" t="n"/>
+      <c r="F68" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G67" s="6" t="inlineStr">
+      <c r="G68" s="6" t="inlineStr">
         <is>
           <t>Respuestas incompletas o no válidas</t>
         </is>
       </c>
-      <c r="H67" s="6" t="inlineStr">
+      <c r="H68" s="6" t="inlineStr">
         <is>
           <t>En caso que falta una respuesta, "Ninguna" se combina con otra opción o se envía un valor fuera de la lista</t>
         </is>
       </c>
-      <c r="I67" s="6" t="inlineStr">
+      <c r="I68" s="6" t="inlineStr">
         <is>
           <t>cuando se intenta guardar</t>
         </is>
       </c>
-      <c r="J67" s="6" t="inlineStr">
+      <c r="J68" s="6" t="inlineStr">
         <is>
           <t>el sistema no guarda e indica qué respuesta corregir</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="55" customHeight="1">
-      <c r="B68" s="20" t="n"/>
-      <c r="C68" s="20" t="n"/>
-      <c r="D68" s="20" t="n"/>
-      <c r="E68" s="20" t="n"/>
-      <c r="F68" s="8" t="n">
+    <row r="69" ht="55" customHeight="1">
+      <c r="B69" s="20" t="n"/>
+      <c r="C69" s="20" t="n"/>
+      <c r="D69" s="20" t="n"/>
+      <c r="E69" s="20" t="n"/>
+      <c r="F69" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G68" s="6" t="inlineStr">
+      <c r="G69" s="6" t="inlineStr">
         <is>
           <t>Confidencialidad</t>
         </is>
       </c>
-      <c r="H68" s="6" t="inlineStr">
+      <c r="H69" s="6" t="inlineStr">
         <is>
           <t>En caso que una petición no tiene sesión válida</t>
         </is>
       </c>
-      <c r="I68" s="6" t="inlineStr">
+      <c r="I69" s="6" t="inlineStr">
         <is>
           <t>cuando intenta consultar o modificar la información de salud</t>
         </is>
       </c>
-      <c r="J68" s="6" t="inlineStr">
+      <c r="J69" s="6" t="inlineStr">
         <is>
           <t>el sistema la rechaza con código 401 sin mostrar datos</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="55" customHeight="1"/>
-    <row r="70" ht="55" customHeight="1">
-      <c r="B70" s="6" t="inlineStr">
+    <row r="70" ht="55" customHeight="1"/>
+    <row r="71" ht="55" customHeight="1">
+      <c r="B71" s="6" t="inlineStr">
         <is>
           <t>FS-HU-20</t>
         </is>
       </c>
-      <c r="C70" s="6" t="inlineStr">
+      <c r="C71" s="6" t="inlineStr">
         <is>
           <t>Como un visitante</t>
         </is>
       </c>
-      <c r="D70" s="6" t="inlineStr">
+      <c r="D71" s="6" t="inlineStr">
         <is>
           <t>Necesito conocer qué ofrece FitSearch antes de crear una cuenta o iniciar sesión</t>
         </is>
       </c>
-      <c r="E70" s="6" t="inlineStr">
+      <c r="E71" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de decidir si registrarme y acceder fácilmente a la plataforma</t>
         </is>
       </c>
-      <c r="F70" s="8" t="n">
+      <c r="F71" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G70" s="6" t="inlineStr">
+      <c r="G71" s="6" t="inlineStr">
         <is>
           <t>Ver la portada sin sesión</t>
         </is>
       </c>
-      <c r="H70" s="6" t="inlineStr">
+      <c r="H71" s="6" t="inlineStr">
         <is>
           <t>En caso que el visitante no ha iniciado sesión</t>
         </is>
       </c>
-      <c r="I70" s="6" t="inlineStr">
+      <c r="I71" s="6" t="inlineStr">
         <is>
           <t>cuando entra a FitSearch</t>
         </is>
       </c>
-      <c r="J70" s="6" t="inlineStr">
+      <c r="J71" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra la portada con lo que ofrece FitSearch (lo disponible y lo próximo) y los accesos "Iniciar sesión" y "Registrarse"</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="55" customHeight="1">
-      <c r="B71" s="22" t="n"/>
-      <c r="C71" s="22" t="n"/>
-      <c r="D71" s="22" t="n"/>
-      <c r="E71" s="22" t="n"/>
-      <c r="F71" s="8" t="n">
+    <row r="72" ht="55" customHeight="1">
+      <c r="B72" s="22" t="n"/>
+      <c r="C72" s="22" t="n"/>
+      <c r="D72" s="22" t="n"/>
+      <c r="E72" s="22" t="n"/>
+      <c r="F72" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G71" s="6" t="inlineStr">
+      <c r="G72" s="6" t="inlineStr">
         <is>
           <t>Con la sesión iniciada</t>
         </is>
       </c>
-      <c r="H71" s="6" t="inlineStr">
+      <c r="H72" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ya inició sesión</t>
         </is>
       </c>
-      <c r="I71" s="6" t="inlineStr">
+      <c r="I72" s="6" t="inlineStr">
         <is>
           <t>cuando intenta abrir la portada</t>
         </is>
       </c>
-      <c r="J71" s="6" t="inlineStr">
+      <c r="J72" s="6" t="inlineStr">
         <is>
           <t>el sistema lo lleva directamente a su Inicio</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="55" customHeight="1">
-      <c r="B72" s="20" t="n"/>
-      <c r="C72" s="20" t="n"/>
-      <c r="D72" s="20" t="n"/>
-      <c r="E72" s="20" t="n"/>
-      <c r="F72" s="8" t="n">
+    <row r="73" ht="55" customHeight="1">
+      <c r="B73" s="20" t="n"/>
+      <c r="C73" s="20" t="n"/>
+      <c r="D73" s="20" t="n"/>
+      <c r="E73" s="20" t="n"/>
+      <c r="F73" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G72" s="6" t="inlineStr">
+      <c r="G73" s="6" t="inlineStr">
         <is>
           <t>Cerrar sesión</t>
         </is>
       </c>
-      <c r="H72" s="6" t="inlineStr">
+      <c r="H73" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario tiene la sesión iniciada</t>
         </is>
       </c>
-      <c r="I72" s="6" t="inlineStr">
+      <c r="I73" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Cerrar sesión"</t>
         </is>
       </c>
-      <c r="J72" s="6" t="inlineStr">
+      <c r="J73" s="6" t="inlineStr">
         <is>
           <t>el sistema cierra la sesión y vuelve a la portada con el mensaje "Cerraste sesión correctamente"</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="55" customHeight="1"/>
-    <row r="74" ht="55" customHeight="1">
-      <c r="B74" s="6" t="inlineStr">
+    <row r="74" ht="55" customHeight="1"/>
+    <row r="75" ht="55" customHeight="1">
+      <c r="B75" s="6" t="inlineStr">
         <is>
           <t>FS-HU-21</t>
         </is>
       </c>
-      <c r="C74" s="6" t="inlineStr">
+      <c r="C75" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D74" s="6" t="inlineStr">
+      <c r="D75" s="6" t="inlineStr">
         <is>
           <t>Necesito un inicio con accesos a las secciones de la plataforma, mi objetivo, mi progreso y mis próximas citas</t>
         </is>
       </c>
-      <c r="E74" s="6" t="inlineStr">
+      <c r="E75" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de orientarme y llegar rápido a lo que necesito</t>
         </is>
       </c>
-      <c r="F74" s="8" t="n">
+      <c r="F75" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G74" s="6" t="inlineStr">
+      <c r="G75" s="6" t="inlineStr">
         <is>
           <t>Llegar al inicio</t>
         </is>
       </c>
-      <c r="H74" s="6" t="inlineStr">
+      <c r="H75" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario inicia sesión y ya eligió su tipo de cuenta</t>
         </is>
       </c>
-      <c r="I74" s="6" t="inlineStr">
+      <c r="I75" s="6" t="inlineStr">
         <is>
           <t>cuando entra a FitSearch o presiona el logo</t>
         </is>
       </c>
-      <c r="J74" s="6" t="inlineStr">
+      <c r="J75" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra el Inicio con accesos rápidos, su objetivo, su meta de calorías, sus próximas citas y profesionales destacados obtenidos de la plataforma</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="55" customHeight="1">
-      <c r="B75" s="22" t="n"/>
-      <c r="C75" s="22" t="n"/>
-      <c r="D75" s="22" t="n"/>
-      <c r="E75" s="22" t="n"/>
-      <c r="F75" s="8" t="n">
+    <row r="76" ht="55" customHeight="1">
+      <c r="B76" s="22" t="n"/>
+      <c r="C76" s="22" t="n"/>
+      <c r="D76" s="22" t="n"/>
+      <c r="E76" s="22" t="n"/>
+      <c r="F76" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G75" s="6" t="inlineStr">
+      <c r="G76" s="6" t="inlineStr">
         <is>
           <t>Sección sin datos</t>
         </is>
       </c>
-      <c r="H75" s="6" t="inlineStr">
+      <c r="H76" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario aún no define su objetivo, no tiene citas o una sección todavía no existe</t>
         </is>
       </c>
-      <c r="I75" s="6" t="inlineStr">
+      <c r="I76" s="6" t="inlineStr">
         <is>
           <t>cuando abre el Inicio o esa sección</t>
         </is>
       </c>
-      <c r="J75" s="6" t="inlineStr">
+      <c r="J76" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra un estado vacío o el aviso "Próximamente" con la acción que corresponde, sin datos inventados</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="55" customHeight="1">
-      <c r="B76" s="20" t="n"/>
-      <c r="C76" s="20" t="n"/>
-      <c r="D76" s="20" t="n"/>
-      <c r="E76" s="20" t="n"/>
-      <c r="F76" s="8" t="n">
+    <row r="77" ht="55" customHeight="1">
+      <c r="B77" s="20" t="n"/>
+      <c r="C77" s="20" t="n"/>
+      <c r="D77" s="20" t="n"/>
+      <c r="E77" s="20" t="n"/>
+      <c r="F77" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G76" s="6" t="inlineStr">
+      <c r="G77" s="6" t="inlineStr">
         <is>
           <t>Menú de la cuenta</t>
         </is>
       </c>
-      <c r="H76" s="6" t="inlineStr">
+      <c r="H77" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario tiene la sesión iniciada</t>
         </is>
       </c>
-      <c r="I76" s="6" t="inlineStr">
+      <c r="I77" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Hola, {nombre}" o su avatar</t>
         </is>
       </c>
-      <c r="J76" s="6" t="inlineStr">
+      <c r="J77" s="6" t="inlineStr">
         <is>
           <t>el sistema abre un menú con "Mi perfil" y "Cerrar sesión"; cerrar sesión vuelve a la portada</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="55" customHeight="1"/>
-    <row r="78" ht="55" customHeight="1">
-      <c r="B78" s="6" t="inlineStr">
+    <row r="78" ht="55" customHeight="1"/>
+    <row r="79" ht="55" customHeight="1">
+      <c r="B79" s="6" t="inlineStr">
         <is>
           <t>FS-HU-22</t>
         </is>
       </c>
-      <c r="C78" s="6" t="inlineStr">
+      <c r="C79" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D78" s="6" t="inlineStr">
+      <c r="D79" s="6" t="inlineStr">
         <is>
           <t>Necesito buscar profesionales por texto y filtrarlos por especialidad, comuna, distancia, calificación y modalidad</t>
         </is>
       </c>
-      <c r="E78" s="6" t="inlineStr">
+      <c r="E79" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de encontrar rápidamente al profesional que se ajusta a lo que busco</t>
         </is>
       </c>
-      <c r="F78" s="8" t="n">
+      <c r="F79" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G78" s="6" t="inlineStr">
+      <c r="G79" s="6" t="inlineStr">
         <is>
           <t>Búsqueda con filtros</t>
         </is>
       </c>
-      <c r="H78" s="6" t="inlineStr">
+      <c r="H79" s="6" t="inlineStr">
         <is>
           <t>En caso que existen profesionales registrados</t>
         </is>
       </c>
-      <c r="I78" s="6" t="inlineStr">
+      <c r="I79" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario busca un texto y elige especialidad, comuna, calificación mínima o modalidad</t>
         </is>
       </c>
-      <c r="J78" s="6" t="inlineStr">
+      <c r="J79" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra solo los profesionales que cumplen los filtros, el total encontrado y el orden elegido</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="55" customHeight="1">
-      <c r="B79" s="22" t="n"/>
-      <c r="C79" s="22" t="n"/>
-      <c r="D79" s="22" t="n"/>
-      <c r="E79" s="22" t="n"/>
-      <c r="F79" s="8" t="n">
+    <row r="80" ht="55" customHeight="1">
+      <c r="B80" s="22" t="n"/>
+      <c r="C80" s="22" t="n"/>
+      <c r="D80" s="22" t="n"/>
+      <c r="E80" s="22" t="n"/>
+      <c r="F80" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G79" s="6" t="inlineStr">
+      <c r="G80" s="6" t="inlineStr">
         <is>
           <t>Búsqueda compartida</t>
         </is>
       </c>
-      <c r="H79" s="6" t="inlineStr">
+      <c r="H80" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario copia la dirección de una búsqueda</t>
         </is>
       </c>
-      <c r="I79" s="6" t="inlineStr">
+      <c r="I80" s="6" t="inlineStr">
         <is>
           <t>cuando otra persona con sesión la abre</t>
         </is>
       </c>
-      <c r="J79" s="6" t="inlineStr">
+      <c r="J80" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra la misma búsqueda con sus filtros, porque quedan guardados en la dirección (nunca la ubicación de la persona)</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="55" customHeight="1">
-      <c r="B80" s="20" t="n"/>
-      <c r="C80" s="20" t="n"/>
-      <c r="D80" s="20" t="n"/>
-      <c r="E80" s="20" t="n"/>
-      <c r="F80" s="8" t="n">
+    <row r="81" ht="55" customHeight="1">
+      <c r="B81" s="20" t="n"/>
+      <c r="C81" s="20" t="n"/>
+      <c r="D81" s="20" t="n"/>
+      <c r="E81" s="20" t="n"/>
+      <c r="F81" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G80" s="6" t="inlineStr">
+      <c r="G81" s="6" t="inlineStr">
         <is>
           <t>Sin coincidencias</t>
         </is>
       </c>
-      <c r="H80" s="6" t="inlineStr">
+      <c r="H81" s="6" t="inlineStr">
         <is>
           <t>En caso que ningún profesional cumple los filtros</t>
         </is>
       </c>
-      <c r="I80" s="6" t="inlineStr">
+      <c r="I81" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario aplica la búsqueda</t>
         </is>
       </c>
-      <c r="J80" s="6" t="inlineStr">
+      <c r="J81" s="6" t="inlineStr">
         <is>
           <t>el sistema indica "No encontramos profesionales con esos filtros" y ofrece limpiar los filtros</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="55" customHeight="1"/>
-    <row r="82" ht="55" customHeight="1">
-      <c r="B82" s="6" t="inlineStr">
+    <row r="82" ht="55" customHeight="1"/>
+    <row r="83" ht="55" customHeight="1">
+      <c r="B83" s="6" t="inlineStr">
         <is>
           <t>FS-HU-23</t>
         </is>
       </c>
-      <c r="C82" s="6" t="inlineStr">
+      <c r="C83" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D82" s="6" t="inlineStr">
+      <c r="D83" s="6" t="inlineStr">
         <is>
           <t>Necesito guardar profesionales como favoritos</t>
         </is>
       </c>
-      <c r="E82" s="6" t="inlineStr">
+      <c r="E83" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de volver a encontrarlos fácilmente</t>
         </is>
       </c>
-      <c r="F82" s="8" t="n">
+      <c r="F83" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G82" s="6" t="inlineStr">
+      <c r="G83" s="6" t="inlineStr">
         <is>
           <t>Guardar un favorito</t>
         </is>
       </c>
-      <c r="H82" s="6" t="inlineStr">
+      <c r="H83" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ve un profesional en el Inicio, el buscador o su ficha</t>
         </is>
       </c>
-      <c r="I82" s="6" t="inlineStr">
+      <c r="I83" s="6" t="inlineStr">
         <is>
           <t>cuando presiona el corazón</t>
         </is>
       </c>
-      <c r="J82" s="6" t="inlineStr">
+      <c r="J83" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda el profesional en sus favoritos y el corazón queda marcado</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="55" customHeight="1">
-      <c r="B83" s="22" t="n"/>
-      <c r="C83" s="22" t="n"/>
-      <c r="D83" s="22" t="n"/>
-      <c r="E83" s="22" t="n"/>
-      <c r="F83" s="8" t="n">
+    <row r="84" ht="55" customHeight="1">
+      <c r="B84" s="22" t="n"/>
+      <c r="C84" s="22" t="n"/>
+      <c r="D84" s="22" t="n"/>
+      <c r="E84" s="22" t="n"/>
+      <c r="F84" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G83" s="6" t="inlineStr">
+      <c r="G84" s="6" t="inlineStr">
         <is>
           <t>Ver favoritos</t>
         </is>
       </c>
-      <c r="H83" s="6" t="inlineStr">
+      <c r="H84" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario guardó profesionales</t>
         </is>
       </c>
-      <c r="I83" s="6" t="inlineStr">
+      <c r="I84" s="6" t="inlineStr">
         <is>
           <t>cuando abre "Favoritos" en el menú</t>
         </is>
       </c>
-      <c r="J83" s="6" t="inlineStr">
+      <c r="J84" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra sus profesionales guardados; si no tiene ninguno, explica cómo guardarlos</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="55" customHeight="1">
-      <c r="B84" s="20" t="n"/>
-      <c r="C84" s="20" t="n"/>
-      <c r="D84" s="20" t="n"/>
-      <c r="E84" s="20" t="n"/>
-      <c r="F84" s="8" t="n">
+    <row r="85" ht="55" customHeight="1">
+      <c r="B85" s="20" t="n"/>
+      <c r="C85" s="20" t="n"/>
+      <c r="D85" s="20" t="n"/>
+      <c r="E85" s="20" t="n"/>
+      <c r="F85" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G84" s="6" t="inlineStr">
+      <c r="G85" s="6" t="inlineStr">
         <is>
           <t>Quitar un favorito</t>
         </is>
       </c>
-      <c r="H84" s="6" t="inlineStr">
+      <c r="H85" s="6" t="inlineStr">
         <is>
           <t>En caso que un profesional está en favoritos</t>
         </is>
       </c>
-      <c r="I84" s="6" t="inlineStr">
+      <c r="I85" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario vuelve a presionar el corazón</t>
         </is>
       </c>
-      <c r="J84" s="6" t="inlineStr">
+      <c r="J85" s="6" t="inlineStr">
         <is>
           <t>el sistema lo quita de sus favoritos</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="55" customHeight="1"/>
-    <row r="86" ht="55" customHeight="1">
-      <c r="B86" s="6" t="inlineStr">
+    <row r="86" ht="55" customHeight="1"/>
+    <row r="87" ht="55" customHeight="1">
+      <c r="B87" s="6" t="inlineStr">
         <is>
           <t>FS-HU-24</t>
         </is>
       </c>
-      <c r="C86" s="6" t="inlineStr">
+      <c r="C87" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D86" s="6" t="inlineStr">
+      <c r="D87" s="6" t="inlineStr">
         <is>
           <t>Necesito calificar con estrellas a un profesional y comentar mi experiencia</t>
         </is>
       </c>
-      <c r="E86" s="6" t="inlineStr">
+      <c r="E87" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de ayudar a otras personas a elegir y conocer la opinión de quienes ya se atendieron</t>
         </is>
       </c>
-      <c r="F86" s="8" t="n">
+      <c r="F87" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G86" s="6" t="inlineStr">
+      <c r="G87" s="6" t="inlineStr">
         <is>
           <t>Publicar una reseña</t>
         </is>
       </c>
-      <c r="H86" s="6" t="inlineStr">
+      <c r="H87" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario abre la ficha de un profesional</t>
         </is>
       </c>
-      <c r="I86" s="6" t="inlineStr">
+      <c r="I87" s="6" t="inlineStr">
         <is>
           <t>cuando elige de 1 a 5 estrellas y, si quiere, escribe un comentario de 10 a 500 caracteres</t>
         </is>
       </c>
-      <c r="J86" s="6" t="inlineStr">
+      <c r="J87" s="6" t="inlineStr">
         <is>
           <t>el sistema publica la reseña con su nombre abreviado y actualiza el promedio y la cantidad de reseñas</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="55" customHeight="1">
-      <c r="B87" s="22" t="n"/>
-      <c r="C87" s="22" t="n"/>
-      <c r="D87" s="22" t="n"/>
-      <c r="E87" s="22" t="n"/>
-      <c r="F87" s="8" t="n">
+    <row r="88" ht="55" customHeight="1">
+      <c r="B88" s="22" t="n"/>
+      <c r="C88" s="22" t="n"/>
+      <c r="D88" s="22" t="n"/>
+      <c r="E88" s="22" t="n"/>
+      <c r="F88" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G87" s="6" t="inlineStr">
+      <c r="G88" s="6" t="inlineStr">
         <is>
           <t>Editar o eliminar su reseña</t>
         </is>
       </c>
-      <c r="H87" s="6" t="inlineStr">
+      <c r="H88" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ya calificó a ese profesional</t>
         </is>
       </c>
-      <c r="I87" s="6" t="inlineStr">
+      <c r="I88" s="6" t="inlineStr">
         <is>
           <t>cuando edita o elimina su reseña</t>
         </is>
       </c>
-      <c r="J87" s="6" t="inlineStr">
+      <c r="J88" s="6" t="inlineStr">
         <is>
           <t>el sistema reemplaza o elimina su única reseña y recalcula el promedio</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="55" customHeight="1">
-      <c r="B88" s="20" t="n"/>
-      <c r="C88" s="20" t="n"/>
-      <c r="D88" s="20" t="n"/>
-      <c r="E88" s="20" t="n"/>
-      <c r="F88" s="8" t="n">
+    <row r="89" ht="55" customHeight="1">
+      <c r="B89" s="20" t="n"/>
+      <c r="C89" s="20" t="n"/>
+      <c r="D89" s="20" t="n"/>
+      <c r="E89" s="20" t="n"/>
+      <c r="F89" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G88" s="6" t="inlineStr">
+      <c r="G89" s="6" t="inlineStr">
         <is>
           <t>Cuenta que no puede calificar</t>
         </is>
       </c>
-      <c r="H88" s="6" t="inlineStr">
+      <c r="H89" s="6" t="inlineStr">
         <is>
           <t>En caso que una cuenta profesional abre una ficha (o la suya propia)</t>
         </is>
       </c>
-      <c r="I88" s="6" t="inlineStr">
+      <c r="I89" s="6" t="inlineStr">
         <is>
           <t>cuando intenta calificar</t>
         </is>
       </c>
-      <c r="J88" s="6" t="inlineStr">
+      <c r="J89" s="6" t="inlineStr">
         <is>
           <t>el sistema le permite leer las reseñas, pero no calificar, y rechaza la calificación si se envía igual</t>
         </is>
       </c>
     </row>
-    <row r="89"/>
-    <row r="90">
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>Nota:</t>
-        </is>
-      </c>
-    </row>
+    <row r="90"/>
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>- Se utilizaron 2 escenarios (criterios de aceptación) por historia de usuario: el caso principal (camino feliz) y un caso de error o borde relevante; FS-HU-14 incluye un tercer escenario para confirmar o cancelar la reserva; FS-HU-15 a FS-HU-24 también incluyen tres escenarios.</t>
+          <t>Nota:</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
+          <t>- Se utilizaron 2 escenarios (criterios de aceptación) por historia de usuario: el caso principal (camino feliz) y un caso de error o borde relevante; FS-HU-14 incluye un tercer escenario para confirmar o cancelar la reserva; FS-HU-15 a FS-HU-24 también incluyen tres escenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" t="inlineStr">
+        <is>
           <t>- El detalle completo de las 24 historias también está disponible en el Product Backlog (PMOInformatica_Plantilla_de_Product_Backlog.xlsx).</t>
         </is>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94"/>
   </sheetData>
   <mergeCells count="98">
+    <mergeCell ref="D75:D77"/>
     <mergeCell ref="B43:B44"/>
+    <mergeCell ref="C51:C53"/>
     <mergeCell ref="G4:J4"/>
+    <mergeCell ref="B55:B57"/>
     <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D55:D57"/>
+    <mergeCell ref="D46:D49"/>
     <mergeCell ref="D9:D11"/>
-    <mergeCell ref="C78:C80"/>
     <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C87:C89"/>
     <mergeCell ref="D13:D14"/>
     <mergeCell ref="D16:D17"/>
     <mergeCell ref="B28:B29"/>
+    <mergeCell ref="E71:E73"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="B37:B38"/>
-    <mergeCell ref="C58:C60"/>
-    <mergeCell ref="E58:E60"/>
-    <mergeCell ref="B62:B64"/>
     <mergeCell ref="C43:C44"/>
-    <mergeCell ref="E82:E84"/>
+    <mergeCell ref="E51:E53"/>
+    <mergeCell ref="C63:C65"/>
     <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C50:C52"/>
-    <mergeCell ref="B70:B72"/>
-    <mergeCell ref="D70:D72"/>
+    <mergeCell ref="C59:C61"/>
+    <mergeCell ref="E59:E61"/>
     <mergeCell ref="E25:E26"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="D34:D35"/>
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="D40:D41"/>
     <mergeCell ref="E13:E14"/>
-    <mergeCell ref="E86:E88"/>
-    <mergeCell ref="B74:B76"/>
-    <mergeCell ref="E62:E64"/>
+    <mergeCell ref="B83:B85"/>
+    <mergeCell ref="D83:D85"/>
     <mergeCell ref="C31:C32"/>
     <mergeCell ref="E31:E32"/>
     <mergeCell ref="C40:C41"/>
-    <mergeCell ref="C62:C64"/>
     <mergeCell ref="E40:E41"/>
-    <mergeCell ref="C54:C56"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="E63:E65"/>
     <mergeCell ref="C4:F4"/>
+    <mergeCell ref="C46:C49"/>
     <mergeCell ref="D25:D26"/>
     <mergeCell ref="D37:D38"/>
-    <mergeCell ref="B46:B48"/>
-    <mergeCell ref="D46:D48"/>
+    <mergeCell ref="C79:C81"/>
+    <mergeCell ref="E79:E81"/>
     <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D86:D88"/>
     <mergeCell ref="C34:C35"/>
     <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C55:C57"/>
+    <mergeCell ref="C71:C73"/>
     <mergeCell ref="C9:C11"/>
     <mergeCell ref="B31:B32"/>
-    <mergeCell ref="E74:E76"/>
     <mergeCell ref="E9:E11"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="D78:D80"/>
-    <mergeCell ref="D74:D76"/>
-    <mergeCell ref="C82:C84"/>
-    <mergeCell ref="D58:D60"/>
-    <mergeCell ref="C66:C68"/>
+    <mergeCell ref="C67:C69"/>
+    <mergeCell ref="B87:B89"/>
+    <mergeCell ref="D87:D89"/>
+    <mergeCell ref="D71:D73"/>
+    <mergeCell ref="B46:B49"/>
     <mergeCell ref="C22:C23"/>
-    <mergeCell ref="E66:E68"/>
+    <mergeCell ref="D67:D69"/>
+    <mergeCell ref="E75:E77"/>
+    <mergeCell ref="B51:B53"/>
     <mergeCell ref="E28:E29"/>
-    <mergeCell ref="B66:B68"/>
-    <mergeCell ref="D82:D84"/>
-    <mergeCell ref="C86:C88"/>
+    <mergeCell ref="D51:D53"/>
+    <mergeCell ref="B63:B65"/>
     <mergeCell ref="B34:B35"/>
-    <mergeCell ref="B50:B52"/>
+    <mergeCell ref="E55:E57"/>
     <mergeCell ref="D28:D29"/>
-    <mergeCell ref="D50:D52"/>
+    <mergeCell ref="B59:B61"/>
+    <mergeCell ref="E46:E49"/>
+    <mergeCell ref="D59:D61"/>
     <mergeCell ref="D43:D44"/>
     <mergeCell ref="E16:E17"/>
-    <mergeCell ref="E78:E80"/>
-    <mergeCell ref="B86:B88"/>
+    <mergeCell ref="E87:E89"/>
     <mergeCell ref="B22:B23"/>
     <mergeCell ref="D31:D32"/>
     <mergeCell ref="D6:D7"/>
-    <mergeCell ref="D62:D64"/>
     <mergeCell ref="E43:E44"/>
-    <mergeCell ref="C70:C72"/>
-    <mergeCell ref="E70:E72"/>
-    <mergeCell ref="E54:E56"/>
     <mergeCell ref="E19:E20"/>
     <mergeCell ref="E34:E35"/>
-    <mergeCell ref="E50:E52"/>
-    <mergeCell ref="B54:B56"/>
-    <mergeCell ref="D54:D56"/>
+    <mergeCell ref="D63:D65"/>
     <mergeCell ref="C25:C26"/>
     <mergeCell ref="E6:E7"/>
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="D79:D81"/>
     <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C74:C76"/>
-    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="C83:C85"/>
+    <mergeCell ref="E83:E85"/>
+    <mergeCell ref="E67:E69"/>
+    <mergeCell ref="B71:B73"/>
     <mergeCell ref="C13:C14"/>
+    <mergeCell ref="B67:B69"/>
     <mergeCell ref="D19:D20"/>
+    <mergeCell ref="C75:C77"/>
     <mergeCell ref="C28:C29"/>
     <mergeCell ref="E22:E23"/>
-    <mergeCell ref="B82:B84"/>
     <mergeCell ref="C37:C38"/>
     <mergeCell ref="B9:B11"/>
     <mergeCell ref="E37:E38"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="E46:E48"/>
-    <mergeCell ref="D66:D68"/>
     <mergeCell ref="D22:D23"/>
   </mergeCells>
   <pageMargins left="0.7086614173228347" right="0.7086614173228347" top="0.7480314960629921" bottom="0.7480314960629921" header="0.3149606299212598" footer="0.3149606299212598"/>

</xml_diff>

<commit_message>
SC-27 y defecto 37: lista y mapa juntos en Profesionales (DAS 1.27)
Lista y mapa lado a lado, detalle bajo el mapa, Ver en el mapa, accesos por especialidad, filtros en barra y opcion de ocultar el mapa. CP-115 a CP-120.
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/Plantilla_Historias_Usuario_con_instructivo.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/Plantilla_Historias_Usuario_con_instructivo.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
     <col width="1.44140625" customWidth="1" style="5" min="1" max="1"/>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Alternar entre mapa y lista</t>
+          <t>Ver la lista y el mapa a la vez</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -1220,20 +1220,20 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>cuando hace clic en el botón de cambiar vista</t>
+          <t>cuando abre Profesionales</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>el sistema alterna entre la vista de mapa y la vista de lista sin perder los resultados</t>
+          <t>el sistema muestra la lista y el mapa juntos (en celular, el mapa arriba de la lista), con un marcador por resultado; si oculta el mapa, ve solo la lista sin perder los resultados ni los filtros (SC-27)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="55" customHeight="1">
-      <c r="B23" s="20" t="n"/>
-      <c r="C23" s="20" t="n"/>
-      <c r="D23" s="20" t="n"/>
-      <c r="E23" s="20" t="n"/>
+      <c r="B23" s="22" t="n"/>
+      <c r="C23" s="22" t="n"/>
+      <c r="D23" s="22" t="n"/>
+      <c r="E23" s="22" t="n"/>
       <c r="F23" s="8" t="n">
         <v>2</v>
       </c>
@@ -1254,667 +1254,667 @@
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>el sistema muestra la tarjeta resumen de ese profesional o establecimiento</t>
+          <t>el sistema muestra bajo el mapa el detalle de ese profesional y marca su tarjeta en la lista (SC-27)</t>
         </is>
       </c>
     </row>
     <row r="24" ht="55" customHeight="1">
-      <c r="B24" s="12" t="n"/>
+      <c r="B24" s="20" t="n"/>
+      <c r="C24" s="20" t="n"/>
+      <c r="D24" s="20" t="n"/>
+      <c r="E24" s="20" t="n"/>
+      <c r="F24" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Ubicar en el mapa un resultado de la lista</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>En caso que el usuario está revisando la lista de resultados</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>cuando presiona «Ver en el mapa» en una tarjeta</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>el sistema lleva el mapa hasta el marcador de ese profesional, lo destaca y muestra su detalle bajo el mapa (SC-27)</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="55" customHeight="1">
-      <c r="B25" s="21" t="inlineStr">
+      <c r="B25" s="12" t="n"/>
+    </row>
+    <row r="26" ht="55" customHeight="1">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>FS-HU-07</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>Necesito conversar con un asistente que me oriente sobre salud y bienestar</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de resolver dudas generales</t>
         </is>
       </c>
-      <c r="F25" s="8" t="n">
+      <c r="F26" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Consulta general de orientación</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario abre el asistente y describe una molestia o duda de salud general</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>cuando envía su mensaje</t>
         </is>
       </c>
-      <c r="J25" s="6" t="inlineStr">
+      <c r="J26" s="6" t="inlineStr">
         <is>
           <t>el sistema responde con orientación general y aclara que no reemplaza a un profesional</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="55" customHeight="1">
-      <c r="B26" s="22" t="n"/>
-      <c r="C26" s="22" t="n"/>
-      <c r="D26" s="22" t="n"/>
-      <c r="E26" s="22" t="n"/>
-      <c r="F26" s="8" t="n">
+    <row r="27" ht="55" customHeight="1">
+      <c r="B27" s="22" t="n"/>
+      <c r="C27" s="22" t="n"/>
+      <c r="D27" s="22" t="n"/>
+      <c r="E27" s="22" t="n"/>
+      <c r="F27" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Continuar una conversación anterior</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario tiene conversaciones previas guardadas</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>cuando selecciona una conversación del historial</t>
         </is>
       </c>
-      <c r="J26" s="6" t="inlineStr">
+      <c r="J27" s="6" t="inlineStr">
         <is>
           <t>el sistema carga el hilo completo y permite seguir conversando desde ahí</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="55" customHeight="1">
-      <c r="B27" s="20" t="n"/>
-      <c r="C27" s="20" t="n"/>
-      <c r="D27" s="20" t="n"/>
-      <c r="E27" s="20" t="n"/>
-      <c r="F27" s="8" t="n">
+    <row r="28" ht="55" customHeight="1">
+      <c r="B28" s="20" t="n"/>
+      <c r="C28" s="20" t="n"/>
+      <c r="D28" s="20" t="n"/>
+      <c r="E28" s="20" t="n"/>
+      <c r="F28" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>Aviso de emergencia solo en situaciones críticas</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario describe una situación crítica (ej. un hueso roto, dificultad para respirar o dolor fuerte en el pecho) o, en cambio, una molestia leve (ej. agujetas o una torcedura leve)</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>cuando envía su mensaje</t>
         </is>
       </c>
-      <c r="J27" s="6" t="inlineStr">
+      <c r="J28" s="6" t="inlineStr">
         <is>
           <t>el sistema indica llamar de inmediato al SAMU (131) solo ante la situación crítica; ante una molestia leve entrega orientación sin ese aviso (SC-26)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="55" customHeight="1"/>
-    <row r="29" ht="55" customHeight="1">
-      <c r="B29" s="6" t="inlineStr">
+    <row r="29" ht="55" customHeight="1"/>
+    <row r="30" ht="55" customHeight="1">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>FS-HU-08</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>Necesito que el asistente me recomiende un tipo de profesional según lo que le cuento</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de saber a quién buscar</t>
         </is>
       </c>
-      <c r="F29" s="8" t="n">
+      <c r="F30" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>Recomendación según síntoma</t>
         </is>
       </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario describe un objetivo o molestia (ej. dolor de rodilla al entrenar)</t>
         </is>
       </c>
-      <c r="I29" s="6" t="inlineStr">
+      <c r="I30" s="6" t="inlineStr">
         <is>
           <t>cuando el asistente identifica la necesidad</t>
         </is>
       </c>
-      <c r="J29" s="6" t="inlineStr">
+      <c r="J30" s="6" t="inlineStr">
         <is>
           <t>el sistema recomienda una categoría de profesional (ej. kinesiólogo) y ofrece buscarlo</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="55" customHeight="1">
-      <c r="B30" s="22" t="n"/>
-      <c r="C30" s="22" t="n"/>
-      <c r="D30" s="22" t="n"/>
-      <c r="E30" s="22" t="n"/>
-      <c r="F30" s="8" t="n">
+    <row r="31" ht="55" customHeight="1">
+      <c r="B31" s="22" t="n"/>
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="22" t="n"/>
+      <c r="E31" s="22" t="n"/>
+      <c r="F31" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>Ir directo a la búsqueda</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>En caso que el asistente ya recomendó una categoría de profesional</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario acepta la sugerencia</t>
         </is>
       </c>
-      <c r="J30" s="6" t="inlineStr">
+      <c r="J31" s="6" t="inlineStr">
         <is>
           <t>el sistema abre el buscador ya filtrado por esa categoría</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="55" customHeight="1">
-      <c r="B31" s="20" t="n"/>
-      <c r="C31" s="20" t="n"/>
-      <c r="D31" s="20" t="n"/>
-      <c r="E31" s="20" t="n"/>
-      <c r="F31" s="8" t="n">
+    <row r="32" ht="55" customHeight="1">
+      <c r="B32" s="20" t="n"/>
+      <c r="C32" s="20" t="n"/>
+      <c r="D32" s="20" t="n"/>
+      <c r="E32" s="20" t="n"/>
+      <c r="F32" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>Sin recomendación cuando no corresponde</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario hace una pregunta general (ej. cómo reservar una hora) o el asistente propone una especialidad que no existe en FitSearch</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr">
+      <c r="I32" s="6" t="inlineStr">
         <is>
           <t>cuando el asistente responde</t>
         </is>
       </c>
-      <c r="J31" s="6" t="inlineStr">
+      <c r="J32" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra la respuesta sin recomendar profesional; solo recomienda especialidades del catálogo de FitSearch (D34)</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="55" customHeight="1"/>
-    <row r="33" ht="55" customHeight="1">
-      <c r="B33" s="6" t="inlineStr">
+    <row r="33" ht="55" customHeight="1"/>
+    <row r="34" ht="55" customHeight="1">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>FS-HU-09</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Necesito registrar lo que como escribiendo en lenguaje natural</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de no tener que llenar formularios manualmente</t>
         </is>
       </c>
-      <c r="F33" s="8" t="n">
+      <c r="F34" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>Registro de una comida completa</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario describe una comida en lenguaje natural (ej. "2 huevos y un plátano")</t>
         </is>
       </c>
-      <c r="I33" s="6" t="inlineStr">
+      <c r="I34" s="6" t="inlineStr">
         <is>
           <t>cuando confirma el registro sugerido por el asistente</t>
         </is>
       </c>
-      <c r="J33" s="6" t="inlineStr">
+      <c r="J34" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda los alimentos, cantidades y la estimación nutricional en el gestor de alimentación</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="55" customHeight="1">
-      <c r="B34" s="20" t="n"/>
-      <c r="C34" s="20" t="n"/>
-      <c r="D34" s="20" t="n"/>
-      <c r="E34" s="20" t="n"/>
-      <c r="F34" s="8" t="n">
+    <row r="35" ht="55" customHeight="1">
+      <c r="B35" s="20" t="n"/>
+      <c r="C35" s="20" t="n"/>
+      <c r="D35" s="20" t="n"/>
+      <c r="E35" s="20" t="n"/>
+      <c r="F35" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G34" s="6" t="inlineStr">
+      <c r="G35" s="6" t="inlineStr">
         <is>
           <t>Alimento no reconocido</t>
         </is>
       </c>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario menciona un alimento que el sistema no logra identificar</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr">
+      <c r="I35" s="6" t="inlineStr">
         <is>
           <t>cuando confirma igualmente el registro</t>
         </is>
       </c>
-      <c r="J34" s="6" t="inlineStr">
+      <c r="J35" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda el resto de los alimentos reconocidos y señala cuál no pudo identificar</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="55" customHeight="1"/>
-    <row r="36" ht="55" customHeight="1">
-      <c r="B36" s="6" t="inlineStr">
+    <row r="36" ht="55" customHeight="1"/>
+    <row r="37" ht="55" customHeight="1">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>FS-HU-10</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Necesito ver mis calorías y macronutrientes consumidos versus mi objetivo diario</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de llevar seguimiento de mi alimentación</t>
         </is>
       </c>
-      <c r="F36" s="8" t="n">
+      <c r="F37" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="G37" s="6" t="inlineStr">
         <is>
           <t>Consulta de progreso diario</t>
         </is>
       </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ya registró comidas durante el día</t>
         </is>
       </c>
-      <c r="I36" s="6" t="inlineStr">
+      <c r="I37" s="6" t="inlineStr">
         <is>
           <t>cuando abre el resumen de calorías y macronutrientes</t>
         </is>
       </c>
-      <c r="J36" s="6" t="inlineStr">
+      <c r="J37" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra el consumo del día comparado con su objetivo diario</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="55" customHeight="1">
-      <c r="B37" s="20" t="n"/>
-      <c r="C37" s="20" t="n"/>
-      <c r="D37" s="20" t="n"/>
-      <c r="E37" s="20" t="n"/>
-      <c r="F37" s="8" t="n">
+    <row r="38" ht="55" customHeight="1">
+      <c r="B38" s="20" t="n"/>
+      <c r="C38" s="20" t="n"/>
+      <c r="D38" s="20" t="n"/>
+      <c r="E38" s="20" t="n"/>
+      <c r="F38" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>Sin registros en el día</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario no ha registrado ninguna comida en el día</t>
         </is>
       </c>
-      <c r="I37" s="6" t="inlineStr">
+      <c r="I38" s="6" t="inlineStr">
         <is>
           <t>cuando abre el resumen de progreso</t>
         </is>
       </c>
-      <c r="J37" s="6" t="inlineStr">
+      <c r="J38" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra el objetivo diario completo como pendiente, sin errores</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="55" customHeight="1"/>
-    <row r="39" ht="55" customHeight="1">
-      <c r="B39" s="6" t="inlineStr">
+    <row r="39" ht="55" customHeight="1"/>
+    <row r="40" ht="55" customHeight="1">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>FS-HU-11</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>Como un equipo de desarrollo</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>Necesito dockerizar la aplicación completa</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de que cualquiera pueda instalarla y ejecutarla fácilmente</t>
         </is>
       </c>
-      <c r="F39" s="8" t="n">
+      <c r="F40" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G39" s="6" t="inlineStr">
+      <c r="G40" s="6" t="inlineStr">
         <is>
           <t>Levantar el entorno completo</t>
         </is>
       </c>
-      <c r="H39" s="6" t="inlineStr">
+      <c r="H40" s="6" t="inlineStr">
         <is>
           <t>En caso que un desarrollador clona el repositorio por primera vez</t>
         </is>
       </c>
-      <c r="I39" s="6" t="inlineStr">
+      <c r="I40" s="6" t="inlineStr">
         <is>
           <t>cuando ejecuta docker-compose up</t>
         </is>
       </c>
-      <c r="J39" s="6" t="inlineStr">
+      <c r="J40" s="6" t="inlineStr">
         <is>
           <t>el sistema levanta frontend, backend y base de datos MySQL correctamente configurados</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="55" customHeight="1">
-      <c r="B40" s="20" t="n"/>
-      <c r="C40" s="20" t="n"/>
-      <c r="D40" s="20" t="n"/>
-      <c r="E40" s="20" t="n"/>
-      <c r="F40" s="8" t="n">
+    <row r="41" ht="55" customHeight="1">
+      <c r="B41" s="20" t="n"/>
+      <c r="C41" s="20" t="n"/>
+      <c r="D41" s="20" t="n"/>
+      <c r="E41" s="20" t="n"/>
+      <c r="F41" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G40" s="6" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>Variables de entorno faltantes</t>
         </is>
       </c>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>En caso que el archivo de variables de entorno no está configurado</t>
         </is>
       </c>
-      <c r="I40" s="6" t="inlineStr">
+      <c r="I41" s="6" t="inlineStr">
         <is>
           <t>cuando se intenta levantar el entorno</t>
         </is>
       </c>
-      <c r="J40" s="6" t="inlineStr">
+      <c r="J41" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra un error claro indicando qué variable falta</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="55" customHeight="1"/>
-    <row r="42" ht="55" customHeight="1">
-      <c r="B42" s="6" t="inlineStr">
+    <row r="42" ht="55" customHeight="1"/>
+    <row r="43" ht="55" customHeight="1">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>FS-HU-12</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>Como un administrador</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Necesito verificar los perfiles de los profesionales</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de que los usuarios identifiquen a los profesionales validados por la plataforma</t>
         </is>
       </c>
-      <c r="F42" s="8" t="n">
+      <c r="F43" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>Verificación de un perfil</t>
         </is>
       </c>
-      <c r="H42" s="6" t="inlineStr">
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>En caso que existe un perfil profesional pendiente de verificación</t>
         </is>
       </c>
-      <c r="I42" s="6" t="inlineStr">
+      <c r="I43" s="6" t="inlineStr">
         <is>
           <t>cuando el administrador lo revisa y lo marca como verificado</t>
         </is>
       </c>
-      <c r="J42" s="6" t="inlineStr">
+      <c r="J43" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda el estado verificado y muestra una insignia de verificación en el perfil y en el listado de profesionales</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="55" customHeight="1">
-      <c r="B43" s="20" t="n"/>
-      <c r="C43" s="20" t="n"/>
-      <c r="D43" s="20" t="n"/>
-      <c r="E43" s="20" t="n"/>
-      <c r="F43" s="8" t="n">
+    <row r="44" ht="55" customHeight="1">
+      <c r="B44" s="20" t="n"/>
+      <c r="C44" s="20" t="n"/>
+      <c r="D44" s="20" t="n"/>
+      <c r="E44" s="20" t="n"/>
+      <c r="F44" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G43" s="6" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
         <is>
           <t>Acceso no autorizado</t>
         </is>
       </c>
-      <c r="H43" s="6" t="inlineStr">
+      <c r="H44" s="6" t="inlineStr">
         <is>
           <t>En caso que un usuario sin rol de administrador intenta verificar un perfil</t>
         </is>
       </c>
-      <c r="I43" s="6" t="inlineStr">
+      <c r="I44" s="6" t="inlineStr">
         <is>
           <t>cuando envía la solicitud de verificación</t>
         </is>
       </c>
-      <c r="J43" s="6" t="inlineStr">
+      <c r="J44" s="6" t="inlineStr">
         <is>
           <t>el sistema rechaza la acción y no modifica el perfil</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="55" customHeight="1"/>
-    <row r="45" ht="55" customHeight="1">
-      <c r="B45" s="6" t="inlineStr">
+    <row r="45" ht="55" customHeight="1"/>
+    <row r="46" ht="55" customHeight="1">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>FS-HU-13</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>Como un profesional</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>Necesito definir mis horarios disponibles</t>
         </is>
       </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de que los usuarios puedan reservar una hora conmigo</t>
         </is>
       </c>
-      <c r="F45" s="8" t="n">
+      <c r="F46" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G45" s="6" t="inlineStr">
+      <c r="G46" s="6" t="inlineStr">
         <is>
           <t>Registrar bloques de disponibilidad</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr">
+      <c r="H46" s="6" t="inlineStr">
         <is>
           <t>En caso que un profesional tiene su perfil creado</t>
         </is>
       </c>
-      <c r="I45" s="6" t="inlineStr">
+      <c r="I46" s="6" t="inlineStr">
         <is>
           <t>cuando agrega un bloque indicando fecha, hora de inicio y hora de término</t>
         </is>
       </c>
-      <c r="J45" s="6" t="inlineStr">
+      <c r="J46" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda el bloque y lo muestra como horario disponible en su perfil</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="55" customHeight="1">
-      <c r="B46" s="20" t="n"/>
-      <c r="C46" s="20" t="n"/>
-      <c r="D46" s="20" t="n"/>
-      <c r="E46" s="20" t="n"/>
-      <c r="F46" s="8" t="n">
+    <row r="47" ht="55" customHeight="1">
+      <c r="B47" s="20" t="n"/>
+      <c r="C47" s="20" t="n"/>
+      <c r="D47" s="20" t="n"/>
+      <c r="E47" s="20" t="n"/>
+      <c r="F47" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G46" s="6" t="inlineStr">
+      <c r="G47" s="6" t="inlineStr">
         <is>
           <t>Bloque inválido o superpuesto</t>
         </is>
       </c>
-      <c r="H46" s="6" t="inlineStr">
+      <c r="H47" s="6" t="inlineStr">
         <is>
           <t>En caso que el profesional ingresa un bloque cuya hora de término no es posterior a la de inicio o que se superpone con otro bloque</t>
         </is>
       </c>
-      <c r="I46" s="6" t="inlineStr">
+      <c r="I47" s="6" t="inlineStr">
         <is>
           <t>cuando intenta guardarlo</t>
         </is>
       </c>
-      <c r="J46" s="6" t="inlineStr">
+      <c r="J47" s="6" t="inlineStr">
         <is>
           <t>el sistema no guarda el bloque e indica el problema</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="55" customHeight="1"/>
-    <row r="48" ht="55" customHeight="1">
-      <c r="B48" s="6" t="inlineStr">
+    <row r="48" ht="55" customHeight="1"/>
+    <row r="49" ht="55" customHeight="1">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>FS-HU-14</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>Necesito reservar una hora con un profesional indicando brevemente lo que necesito</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de agendar una atención que se ajuste a mi necesidad</t>
         </is>
       </c>
-      <c r="F48" s="8" t="n">
+      <c r="F49" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G48" s="6" t="inlineStr">
+      <c r="G49" s="6" t="inlineStr">
         <is>
           <t>Reserva con mensaje</t>
         </is>
       </c>
-      <c r="H48" s="6" t="inlineStr">
+      <c r="H49" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ve un horario disponible en el perfil de un profesional</t>
         </is>
       </c>
-      <c r="I48" s="6" t="inlineStr">
+      <c r="I49" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Reservar", escribe un mensaje breve con lo que necesita y confirma</t>
         </is>
       </c>
-      <c r="J48" s="6" t="inlineStr">
+      <c r="J49" s="6" t="inlineStr">
         <is>
           <t>el sistema crea la reserva en estado pendiente, el horario deja de estar disponible y el profesional ve la reserva junto al mensaje</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="55" customHeight="1">
-      <c r="B49" s="22" t="n"/>
-      <c r="C49" s="22" t="n"/>
-      <c r="D49" s="22" t="n"/>
-      <c r="E49" s="22" t="n"/>
-      <c r="F49" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>Reserva sin mensaje u horario ocupado</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>En caso que el usuario no escribe el mensaje o el horario fue tomado por otro usuario</t>
-        </is>
-      </c>
-      <c r="I49" s="6" t="inlineStr">
-        <is>
-          <t>cuando intenta confirmar la reserva</t>
-        </is>
-      </c>
-      <c r="J49" s="6" t="inlineStr">
-        <is>
-          <t>el sistema no crea la reserva e indica que debe escribir el mensaje o elegir otro horario</t>
         </is>
       </c>
     </row>
@@ -1924,1222 +1924,1251 @@
       <c r="D50" s="22" t="n"/>
       <c r="E50" s="22" t="n"/>
       <c r="F50" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>Reserva sin mensaje u horario ocupado</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>En caso que el usuario no escribe el mensaje o el horario fue tomado por otro usuario</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>cuando intenta confirmar la reserva</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="inlineStr">
+        <is>
+          <t>el sistema no crea la reserva e indica que debe escribir el mensaje o elegir otro horario</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="55" customHeight="1">
+      <c r="B51" s="22" t="n"/>
+      <c r="C51" s="22" t="n"/>
+      <c r="D51" s="22" t="n"/>
+      <c r="E51" s="22" t="n"/>
+      <c r="F51" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G50" s="6" t="inlineStr">
+      <c r="G51" s="6" t="inlineStr">
         <is>
           <t>Confirmar o cancelar una reserva</t>
         </is>
       </c>
-      <c r="H50" s="6" t="inlineStr">
+      <c r="H51" s="6" t="inlineStr">
         <is>
           <t>En caso que existe una reserva pendiente</t>
         </is>
       </c>
-      <c r="I50" s="6" t="inlineStr">
+      <c r="I51" s="6" t="inlineStr">
         <is>
           <t>cuando el profesional la confirma o cualquiera de las partes la cancela</t>
         </is>
       </c>
-      <c r="J50" s="6" t="inlineStr">
+      <c r="J51" s="6" t="inlineStr">
         <is>
           <t>el sistema actualiza el estado, libera el horario si se cancela y ambas partes ven el estado actualizado</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="55" customHeight="1">
-      <c r="B51" s="20" t="n"/>
-      <c r="C51" s="20" t="n"/>
-      <c r="D51" s="20" t="n"/>
-      <c r="E51" s="20" t="n"/>
-      <c r="F51" s="8" t="inlineStr">
+    <row r="52" ht="55" customHeight="1">
+      <c r="B52" s="20" t="n"/>
+      <c r="C52" s="20" t="n"/>
+      <c r="D52" s="20" t="n"/>
+      <c r="E52" s="20" t="n"/>
+      <c r="F52" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G51" s="6" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>Límite de una reserva activa por profesional</t>
         </is>
       </c>
-      <c r="H51" s="6" t="inlineStr">
+      <c r="H52" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ya tiene una reserva pendiente o confirmada para un horario futuro con ese profesional</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr">
+      <c r="I52" s="6" t="inlineStr">
         <is>
           <t>cuando intenta reservar otra hora con el mismo profesional</t>
         </is>
       </c>
-      <c r="J51" s="6" t="inlineStr">
+      <c r="J52" s="6" t="inlineStr">
         <is>
           <t>el sistema no crea la reserva, se lo avisa antes de escribir el mensaje y le indica que primero cancele la reserva activa en "Mis citas"; las citas que ya pasaron no cuentan para este límite (decisión del Product Owner del 12-10-2026)</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="55" customHeight="1"/>
-    <row r="53" ht="55" customHeight="1">
-      <c r="B53" s="6" t="inlineStr">
+    <row r="53" ht="55" customHeight="1"/>
+    <row r="54" ht="55" customHeight="1">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>FS-HU-15</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>Necesito recuperar mi contraseña mediante un enlace enviado a mi correo</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de volver a acceder a mi cuenta si la olvido</t>
         </is>
       </c>
-      <c r="F53" s="8" t="n">
+      <c r="F54" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="G54" s="6" t="inlineStr">
         <is>
           <t>Solicitar enlace de recuperación</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr">
+      <c r="H54" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario olvidó su contraseña</t>
         </is>
       </c>
-      <c r="I53" s="6" t="inlineStr">
+      <c r="I54" s="6" t="inlineStr">
         <is>
           <t>cuando escribe su correo en "¿Olvidaste tu contraseña?" y presiona "Enviar enlace"</t>
         </is>
       </c>
-      <c r="J53" s="6" t="inlineStr">
+      <c r="J54" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra siempre el mismo mensaje de confirmación y, si el correo está registrado, envía un correo con un enlace válido por 60 minutos</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="55" customHeight="1">
-      <c r="B54" s="22" t="n"/>
-      <c r="C54" s="22" t="n"/>
-      <c r="D54" s="22" t="n"/>
-      <c r="E54" s="22" t="n"/>
-      <c r="F54" s="8" t="n">
+    <row r="55" ht="55" customHeight="1">
+      <c r="B55" s="22" t="n"/>
+      <c r="C55" s="22" t="n"/>
+      <c r="D55" s="22" t="n"/>
+      <c r="E55" s="22" t="n"/>
+      <c r="F55" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G54" s="6" t="inlineStr">
+      <c r="G55" s="6" t="inlineStr">
         <is>
           <t>Restablecer la contraseña</t>
         </is>
       </c>
-      <c r="H54" s="6" t="inlineStr">
+      <c r="H55" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario abre un enlace de recuperación vigente</t>
         </is>
       </c>
-      <c r="I54" s="6" t="inlineStr">
+      <c r="I55" s="6" t="inlineStr">
         <is>
           <t>cuando escribe una contraseña nueva de al menos 8 caracteres y su confirmación coincide</t>
         </is>
       </c>
-      <c r="J54" s="6" t="inlineStr">
+      <c r="J55" s="6" t="inlineStr">
         <is>
           <t>el sistema actualiza la contraseña, inutiliza el enlace y permite iniciar sesión con la contraseña nueva</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="55" customHeight="1">
-      <c r="B55" s="20" t="n"/>
-      <c r="C55" s="20" t="n"/>
-      <c r="D55" s="20" t="n"/>
-      <c r="E55" s="20" t="n"/>
-      <c r="F55" s="8" t="n">
+    <row r="56" ht="55" customHeight="1">
+      <c r="B56" s="20" t="n"/>
+      <c r="C56" s="20" t="n"/>
+      <c r="D56" s="20" t="n"/>
+      <c r="E56" s="20" t="n"/>
+      <c r="F56" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G55" s="6" t="inlineStr">
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>Enlace vencido o usado</t>
         </is>
       </c>
-      <c r="H55" s="6" t="inlineStr">
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>En caso que el enlace ya venció, ya se usó o fue alterado</t>
         </is>
       </c>
-      <c r="I55" s="6" t="inlineStr">
+      <c r="I56" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario intenta restablecer la contraseña</t>
         </is>
       </c>
-      <c r="J55" s="6" t="inlineStr">
+      <c r="J56" s="6" t="inlineStr">
         <is>
           <t>el sistema no cambia la contraseña e indica que debe solicitar un enlace nuevo</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="55" customHeight="1"/>
-    <row r="57" ht="55" customHeight="1">
-      <c r="B57" s="6" t="inlineStr">
+    <row r="57" ht="55" customHeight="1"/>
+    <row r="58" ht="55" customHeight="1">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>FS-HU-16</t>
         </is>
       </c>
-      <c r="C57" s="6" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>Como un usuario o profesional</t>
         </is>
       </c>
-      <c r="D57" s="6" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>Necesito registrarme e iniciar sesión con mi cuenta de Google</t>
         </is>
       </c>
-      <c r="E57" s="6" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de acceder sin crear ni recordar otra contraseña</t>
         </is>
       </c>
-      <c r="F57" s="8" t="n">
+      <c r="F58" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G57" s="6" t="inlineStr">
+      <c r="G58" s="6" t="inlineStr">
         <is>
           <t>Primer acceso con Google</t>
         </is>
       </c>
-      <c r="H57" s="6" t="inlineStr">
+      <c r="H58" s="6" t="inlineStr">
         <is>
           <t>En caso que la persona no tiene cuenta en FitSearch</t>
         </is>
       </c>
-      <c r="I57" s="6" t="inlineStr">
+      <c r="I58" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Continuar con Google" y autoriza el acceso</t>
         </is>
       </c>
-      <c r="J57" s="6" t="inlineStr">
+      <c r="J58" s="6" t="inlineStr">
         <is>
           <t>el sistema crea la cuenta y su perfil vacío, deja la sesión iniciada y le pide elegir su tipo de cuenta en el primer paso del perfil</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="55" customHeight="1">
-      <c r="B58" s="22" t="n"/>
-      <c r="C58" s="22" t="n"/>
-      <c r="D58" s="22" t="n"/>
-      <c r="E58" s="22" t="n"/>
-      <c r="F58" s="8" t="n">
+    <row r="59" ht="55" customHeight="1">
+      <c r="B59" s="22" t="n"/>
+      <c r="C59" s="22" t="n"/>
+      <c r="D59" s="22" t="n"/>
+      <c r="E59" s="22" t="n"/>
+      <c r="F59" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G58" s="6" t="inlineStr">
+      <c r="G59" s="6" t="inlineStr">
         <is>
           <t>Cuenta existente con el mismo correo</t>
         </is>
       </c>
-      <c r="H58" s="6" t="inlineStr">
+      <c r="H59" s="6" t="inlineStr">
         <is>
           <t>En caso que ya existe una cuenta registrada con el correo de Google</t>
         </is>
       </c>
-      <c r="I58" s="6" t="inlineStr">
+      <c r="I59" s="6" t="inlineStr">
         <is>
           <t>cuando la persona continúa con Google</t>
         </is>
       </c>
-      <c r="J58" s="6" t="inlineStr">
+      <c r="J59" s="6" t="inlineStr">
         <is>
           <t>el sistema vincula la cuenta de Google a la cuenta existente e inicia la sesión sin crear un usuario duplicado</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="55" customHeight="1">
-      <c r="B59" s="20" t="n"/>
-      <c r="C59" s="20" t="n"/>
-      <c r="D59" s="20" t="n"/>
-      <c r="E59" s="20" t="n"/>
-      <c r="F59" s="8" t="n">
+    <row r="60" ht="55" customHeight="1">
+      <c r="B60" s="20" t="n"/>
+      <c r="C60" s="20" t="n"/>
+      <c r="D60" s="20" t="n"/>
+      <c r="E60" s="20" t="n"/>
+      <c r="F60" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G59" s="6" t="inlineStr">
+      <c r="G60" s="6" t="inlineStr">
         <is>
           <t>Acceso con Google inválido</t>
         </is>
       </c>
-      <c r="H59" s="6" t="inlineStr">
+      <c r="H60" s="6" t="inlineStr">
         <is>
           <t>En caso que la validación de Google falla o el correo no está verificado</t>
         </is>
       </c>
-      <c r="I59" s="6" t="inlineStr">
+      <c r="I60" s="6" t="inlineStr">
         <is>
           <t>cuando el sistema recibe la solicitud de acceso</t>
         </is>
       </c>
-      <c r="J59" s="6" t="inlineStr">
+      <c r="J60" s="6" t="inlineStr">
         <is>
           <t>el sistema rechaza el acceso y muestra un mensaje de error sin crear la cuenta</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="55" customHeight="1"/>
-    <row r="61" ht="55" customHeight="1">
-      <c r="B61" s="6" t="inlineStr">
+    <row r="61" ht="55" customHeight="1"/>
+    <row r="62" ht="55" customHeight="1">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>FS-HU-17</t>
         </is>
       </c>
-      <c r="C61" s="6" t="inlineStr">
+      <c r="C62" s="6" t="inlineStr">
         <is>
           <t>Como un usuario o profesional</t>
         </is>
       </c>
-      <c r="D61" s="6" t="inlineStr">
+      <c r="D62" s="6" t="inlineStr">
         <is>
           <t>Necesito confirmar mi contraseña al registrarme y decidir si mantener mi sesión iniciada</t>
         </is>
       </c>
-      <c r="E61" s="6" t="inlineStr">
+      <c r="E62" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de acceder a las funciones que me corresponden de forma cómoda y segura</t>
         </is>
       </c>
-      <c r="F61" s="8" t="n">
+      <c r="F62" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G61" s="6" t="inlineStr">
+      <c r="G62" s="6" t="inlineStr">
         <is>
           <t>Registro sin elegir rol</t>
         </is>
       </c>
-      <c r="H61" s="6" t="inlineStr">
+      <c r="H62" s="6" t="inlineStr">
         <is>
           <t>En caso que la persona completa el formulario de registro</t>
         </is>
       </c>
-      <c r="I61" s="6" t="inlineStr">
+      <c r="I62" s="6" t="inlineStr">
         <is>
           <t>cuando confirma el registro</t>
         </is>
       </c>
-      <c r="J61" s="6" t="inlineStr">
+      <c r="J62" s="6" t="inlineStr">
         <is>
           <t>el sistema crea la cuenta como usuario y le pide elegir su tipo de cuenta en el perfil; nunca permite registrarse como administrador</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="55" customHeight="1">
-      <c r="B62" s="22" t="n"/>
-      <c r="C62" s="22" t="n"/>
-      <c r="D62" s="22" t="n"/>
-      <c r="E62" s="22" t="n"/>
-      <c r="F62" s="8" t="n">
+    <row r="63" ht="55" customHeight="1">
+      <c r="B63" s="22" t="n"/>
+      <c r="C63" s="22" t="n"/>
+      <c r="D63" s="22" t="n"/>
+      <c r="E63" s="22" t="n"/>
+      <c r="F63" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G62" s="6" t="inlineStr">
+      <c r="G63" s="6" t="inlineStr">
         <is>
           <t>Contraseñas distintas</t>
         </is>
       </c>
-      <c r="H62" s="6" t="inlineStr">
+      <c r="H63" s="6" t="inlineStr">
         <is>
           <t>En caso que la contraseña y su confirmación no coinciden</t>
         </is>
       </c>
-      <c r="I62" s="6" t="inlineStr">
+      <c r="I63" s="6" t="inlineStr">
         <is>
           <t>cuando la persona intenta registrarse</t>
         </is>
       </c>
-      <c r="J62" s="6" t="inlineStr">
+      <c r="J63" s="6" t="inlineStr">
         <is>
           <t>el sistema no crea la cuenta e indica que las contraseñas no coinciden</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="55" customHeight="1">
-      <c r="B63" s="20" t="n"/>
-      <c r="C63" s="20" t="n"/>
-      <c r="D63" s="20" t="n"/>
-      <c r="E63" s="20" t="n"/>
-      <c r="F63" s="8" t="n">
+    <row r="64" ht="55" customHeight="1">
+      <c r="B64" s="20" t="n"/>
+      <c r="C64" s="20" t="n"/>
+      <c r="D64" s="20" t="n"/>
+      <c r="E64" s="20" t="n"/>
+      <c r="F64" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G63" s="6" t="inlineStr">
+      <c r="G64" s="6" t="inlineStr">
         <is>
           <t>Recordarme</t>
         </is>
       </c>
-      <c r="H63" s="6" t="inlineStr">
+      <c r="H64" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario inicia sesión</t>
         </is>
       </c>
-      <c r="I63" s="6" t="inlineStr">
+      <c r="I64" s="6" t="inlineStr">
         <is>
           <t>cuando marca o no marca "Recordarme"</t>
         </is>
       </c>
-      <c r="J63" s="6" t="inlineStr">
+      <c r="J64" s="6" t="inlineStr">
         <is>
           <t>si lo marcó, la sesión se mantiene hasta 30 días aunque cierre el navegador; si no, la sesión termina al cerrar el navegador</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="55" customHeight="1"/>
-    <row r="65" ht="55" customHeight="1">
-      <c r="B65" s="6" t="inlineStr">
+    <row r="65" ht="55" customHeight="1"/>
+    <row r="66" ht="55" customHeight="1">
+      <c r="B66" s="6" t="inlineStr">
         <is>
           <t>FS-HU-18</t>
         </is>
       </c>
-      <c r="C65" s="6" t="inlineStr">
+      <c r="C66" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D65" s="6" t="inlineStr">
+      <c r="D66" s="6" t="inlineStr">
         <is>
           <t>Necesito indicar mi objetivo principal y mi estilo de vida (comidas al día y horas de sueño)</t>
         </is>
       </c>
-      <c r="E65" s="6" t="inlineStr">
+      <c r="E66" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de recibir una orientación acorde a lo que busco lograr</t>
         </is>
       </c>
-      <c r="F65" s="8" t="n">
+      <c r="F66" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G65" s="6" t="inlineStr">
+      <c r="G66" s="6" t="inlineStr">
         <is>
           <t>Guardar objetivos y estilo de vida</t>
         </is>
       </c>
-      <c r="H65" s="6" t="inlineStr">
+      <c r="H66" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario completó sus datos personales en el asistente</t>
         </is>
       </c>
-      <c r="I65" s="6" t="inlineStr">
+      <c r="I66" s="6" t="inlineStr">
         <is>
           <t>cuando elige su objetivo principal, las comidas al día y las horas de sueño y presiona "Siguiente"</t>
         </is>
       </c>
-      <c r="J65" s="6" t="inlineStr">
+      <c r="J66" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda la información y avanza al paso de información de salud</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="55" customHeight="1">
-      <c r="B66" s="22" t="n"/>
-      <c r="C66" s="22" t="n"/>
-      <c r="D66" s="22" t="n"/>
-      <c r="E66" s="22" t="n"/>
-      <c r="F66" s="8" t="n">
+    <row r="67" ht="55" customHeight="1">
+      <c r="B67" s="22" t="n"/>
+      <c r="C67" s="22" t="n"/>
+      <c r="D67" s="22" t="n"/>
+      <c r="E67" s="22" t="n"/>
+      <c r="F67" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G66" s="6" t="inlineStr">
+      <c r="G67" s="6" t="inlineStr">
         <is>
           <t>Datos incompletos</t>
         </is>
       </c>
-      <c r="H66" s="6" t="inlineStr">
+      <c r="H67" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario no responde alguna de las preguntas</t>
         </is>
       </c>
-      <c r="I66" s="6" t="inlineStr">
+      <c r="I67" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Siguiente"</t>
         </is>
       </c>
-      <c r="J66" s="6" t="inlineStr">
+      <c r="J67" s="6" t="inlineStr">
         <is>
           <t>el sistema no guarda y señala cada pregunta pendiente</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="55" customHeight="1">
-      <c r="B67" s="20" t="n"/>
-      <c r="C67" s="20" t="n"/>
-      <c r="D67" s="20" t="n"/>
-      <c r="E67" s="20" t="n"/>
-      <c r="F67" s="8" t="n">
+    <row r="68" ht="55" customHeight="1">
+      <c r="B68" s="20" t="n"/>
+      <c r="C68" s="20" t="n"/>
+      <c r="D68" s="20" t="n"/>
+      <c r="E68" s="20" t="n"/>
+      <c r="F68" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G67" s="6" t="inlineStr">
+      <c r="G68" s="6" t="inlineStr">
         <is>
           <t>Editar desde el resumen</t>
         </is>
       </c>
-      <c r="H67" s="6" t="inlineStr">
+      <c r="H68" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ya completó su perfil</t>
         </is>
       </c>
-      <c r="I67" s="6" t="inlineStr">
+      <c r="I68" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Editar" en Objetivos y estilo de vida, cambia su objetivo y guarda</t>
         </is>
       </c>
-      <c r="J67" s="6" t="inlineStr">
+      <c r="J68" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda el cambio y vuelve al resumen mostrando el objetivo actualizado</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="55" customHeight="1"/>
-    <row r="69" ht="55" customHeight="1">
-      <c r="B69" s="6" t="inlineStr">
+    <row r="69" ht="55" customHeight="1"/>
+    <row r="70" ht="55" customHeight="1">
+      <c r="B70" s="6" t="inlineStr">
         <is>
           <t>FS-HU-19</t>
         </is>
       </c>
-      <c r="C69" s="6" t="inlineStr">
+      <c r="C70" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D69" s="6" t="inlineStr">
+      <c r="D70" s="6" t="inlineStr">
         <is>
           <t>Necesito registrar mis condiciones médicas, medicamentos y alergias de forma confidencial</t>
         </is>
       </c>
-      <c r="E69" s="6" t="inlineStr">
+      <c r="E70" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de recibir recomendaciones más seguras y adecuadas a mi situación</t>
         </is>
       </c>
-      <c r="F69" s="8" t="n">
+      <c r="F70" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G69" s="6" t="inlineStr">
+      <c r="G70" s="6" t="inlineStr">
         <is>
           <t>Guardar información de salud</t>
         </is>
       </c>
-      <c r="H69" s="6" t="inlineStr">
+      <c r="H70" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario está en el paso de información de salud</t>
         </is>
       </c>
-      <c r="I69" s="6" t="inlineStr">
+      <c r="I70" s="6" t="inlineStr">
         <is>
           <t>cuando marca sus condiciones médicas, indica si toma medicamentos (y de qué tipo) y sus alergias, y presiona "Siguiente"</t>
         </is>
       </c>
-      <c r="J69" s="6" t="inlineStr">
+      <c r="J70" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda la información, muestra "¡Información guardada!" con el requerimiento calórico estimado y luego el resumen del perfil</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="55" customHeight="1">
-      <c r="B70" s="22" t="n"/>
-      <c r="C70" s="22" t="n"/>
-      <c r="D70" s="22" t="n"/>
-      <c r="E70" s="22" t="n"/>
-      <c r="F70" s="8" t="n">
+    <row r="71" ht="55" customHeight="1">
+      <c r="B71" s="22" t="n"/>
+      <c r="C71" s="22" t="n"/>
+      <c r="D71" s="22" t="n"/>
+      <c r="E71" s="22" t="n"/>
+      <c r="F71" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G70" s="6" t="inlineStr">
+      <c r="G71" s="6" t="inlineStr">
         <is>
           <t>Respuestas incompletas o no válidas</t>
         </is>
       </c>
-      <c r="H70" s="6" t="inlineStr">
+      <c r="H71" s="6" t="inlineStr">
         <is>
           <t>En caso que falta una respuesta, "Ninguna" se combina con otra opción o se envía un valor fuera de la lista</t>
         </is>
       </c>
-      <c r="I70" s="6" t="inlineStr">
+      <c r="I71" s="6" t="inlineStr">
         <is>
           <t>cuando se intenta guardar</t>
         </is>
       </c>
-      <c r="J70" s="6" t="inlineStr">
+      <c r="J71" s="6" t="inlineStr">
         <is>
           <t>el sistema no guarda e indica qué respuesta corregir</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="55" customHeight="1">
-      <c r="B71" s="20" t="n"/>
-      <c r="C71" s="20" t="n"/>
-      <c r="D71" s="20" t="n"/>
-      <c r="E71" s="20" t="n"/>
-      <c r="F71" s="8" t="n">
+    <row r="72" ht="55" customHeight="1">
+      <c r="B72" s="20" t="n"/>
+      <c r="C72" s="20" t="n"/>
+      <c r="D72" s="20" t="n"/>
+      <c r="E72" s="20" t="n"/>
+      <c r="F72" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G71" s="6" t="inlineStr">
+      <c r="G72" s="6" t="inlineStr">
         <is>
           <t>Confidencialidad</t>
         </is>
       </c>
-      <c r="H71" s="6" t="inlineStr">
+      <c r="H72" s="6" t="inlineStr">
         <is>
           <t>En caso que una petición no tiene sesión válida</t>
         </is>
       </c>
-      <c r="I71" s="6" t="inlineStr">
+      <c r="I72" s="6" t="inlineStr">
         <is>
           <t>cuando intenta consultar o modificar la información de salud</t>
         </is>
       </c>
-      <c r="J71" s="6" t="inlineStr">
+      <c r="J72" s="6" t="inlineStr">
         <is>
           <t>el sistema la rechaza con código 401 sin mostrar datos</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="55" customHeight="1"/>
-    <row r="73" ht="55" customHeight="1">
-      <c r="B73" s="6" t="inlineStr">
+    <row r="73" ht="55" customHeight="1"/>
+    <row r="74" ht="55" customHeight="1">
+      <c r="B74" s="6" t="inlineStr">
         <is>
           <t>FS-HU-20</t>
         </is>
       </c>
-      <c r="C73" s="6" t="inlineStr">
+      <c r="C74" s="6" t="inlineStr">
         <is>
           <t>Como un visitante</t>
         </is>
       </c>
-      <c r="D73" s="6" t="inlineStr">
+      <c r="D74" s="6" t="inlineStr">
         <is>
           <t>Necesito conocer qué ofrece FitSearch antes de crear una cuenta o iniciar sesión</t>
         </is>
       </c>
-      <c r="E73" s="6" t="inlineStr">
+      <c r="E74" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de decidir si registrarme y acceder fácilmente a la plataforma</t>
         </is>
       </c>
-      <c r="F73" s="8" t="n">
+      <c r="F74" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G73" s="6" t="inlineStr">
+      <c r="G74" s="6" t="inlineStr">
         <is>
           <t>Ver la portada sin sesión</t>
         </is>
       </c>
-      <c r="H73" s="6" t="inlineStr">
+      <c r="H74" s="6" t="inlineStr">
         <is>
           <t>En caso que el visitante no ha iniciado sesión</t>
         </is>
       </c>
-      <c r="I73" s="6" t="inlineStr">
+      <c r="I74" s="6" t="inlineStr">
         <is>
           <t>cuando entra a FitSearch</t>
         </is>
       </c>
-      <c r="J73" s="6" t="inlineStr">
+      <c r="J74" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra la portada con lo que ofrece FitSearch (lo disponible y lo próximo) y los accesos "Iniciar sesión" y "Registrarse"</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="55" customHeight="1">
-      <c r="B74" s="22" t="n"/>
-      <c r="C74" s="22" t="n"/>
-      <c r="D74" s="22" t="n"/>
-      <c r="E74" s="22" t="n"/>
-      <c r="F74" s="8" t="n">
+    <row r="75" ht="55" customHeight="1">
+      <c r="B75" s="22" t="n"/>
+      <c r="C75" s="22" t="n"/>
+      <c r="D75" s="22" t="n"/>
+      <c r="E75" s="22" t="n"/>
+      <c r="F75" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G74" s="6" t="inlineStr">
+      <c r="G75" s="6" t="inlineStr">
         <is>
           <t>Con la sesión iniciada</t>
         </is>
       </c>
-      <c r="H74" s="6" t="inlineStr">
+      <c r="H75" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ya inició sesión</t>
         </is>
       </c>
-      <c r="I74" s="6" t="inlineStr">
+      <c r="I75" s="6" t="inlineStr">
         <is>
           <t>cuando intenta abrir la portada</t>
         </is>
       </c>
-      <c r="J74" s="6" t="inlineStr">
+      <c r="J75" s="6" t="inlineStr">
         <is>
           <t>el sistema lo lleva directamente a su Inicio</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="55" customHeight="1">
-      <c r="B75" s="20" t="n"/>
-      <c r="C75" s="20" t="n"/>
-      <c r="D75" s="20" t="n"/>
-      <c r="E75" s="20" t="n"/>
-      <c r="F75" s="8" t="n">
+    <row r="76" ht="55" customHeight="1">
+      <c r="B76" s="20" t="n"/>
+      <c r="C76" s="20" t="n"/>
+      <c r="D76" s="20" t="n"/>
+      <c r="E76" s="20" t="n"/>
+      <c r="F76" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G75" s="6" t="inlineStr">
+      <c r="G76" s="6" t="inlineStr">
         <is>
           <t>Cerrar sesión</t>
         </is>
       </c>
-      <c r="H75" s="6" t="inlineStr">
+      <c r="H76" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario tiene la sesión iniciada</t>
         </is>
       </c>
-      <c r="I75" s="6" t="inlineStr">
+      <c r="I76" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Cerrar sesión"</t>
         </is>
       </c>
-      <c r="J75" s="6" t="inlineStr">
+      <c r="J76" s="6" t="inlineStr">
         <is>
           <t>el sistema cierra la sesión y vuelve a la portada con el mensaje "Cerraste sesión correctamente"</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="55" customHeight="1"/>
-    <row r="77" ht="55" customHeight="1">
-      <c r="B77" s="6" t="inlineStr">
+    <row r="77" ht="55" customHeight="1"/>
+    <row r="78" ht="55" customHeight="1">
+      <c r="B78" s="6" t="inlineStr">
         <is>
           <t>FS-HU-21</t>
         </is>
       </c>
-      <c r="C77" s="6" t="inlineStr">
+      <c r="C78" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D77" s="6" t="inlineStr">
+      <c r="D78" s="6" t="inlineStr">
         <is>
           <t>Necesito un inicio con accesos a las secciones de la plataforma, mi objetivo, mi progreso y mis próximas citas</t>
         </is>
       </c>
-      <c r="E77" s="6" t="inlineStr">
+      <c r="E78" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de orientarme y llegar rápido a lo que necesito</t>
         </is>
       </c>
-      <c r="F77" s="8" t="n">
+      <c r="F78" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G77" s="6" t="inlineStr">
+      <c r="G78" s="6" t="inlineStr">
         <is>
           <t>Llegar al inicio</t>
         </is>
       </c>
-      <c r="H77" s="6" t="inlineStr">
+      <c r="H78" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario inicia sesión y ya eligió su tipo de cuenta</t>
         </is>
       </c>
-      <c r="I77" s="6" t="inlineStr">
+      <c r="I78" s="6" t="inlineStr">
         <is>
           <t>cuando entra a FitSearch o presiona el logo</t>
         </is>
       </c>
-      <c r="J77" s="6" t="inlineStr">
+      <c r="J78" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra el Inicio con accesos rápidos, su objetivo, su meta de calorías, sus próximas citas y profesionales destacados obtenidos de la plataforma</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="55" customHeight="1">
-      <c r="B78" s="22" t="n"/>
-      <c r="C78" s="22" t="n"/>
-      <c r="D78" s="22" t="n"/>
-      <c r="E78" s="22" t="n"/>
-      <c r="F78" s="8" t="n">
+    <row r="79" ht="55" customHeight="1">
+      <c r="B79" s="22" t="n"/>
+      <c r="C79" s="22" t="n"/>
+      <c r="D79" s="22" t="n"/>
+      <c r="E79" s="22" t="n"/>
+      <c r="F79" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G78" s="6" t="inlineStr">
+      <c r="G79" s="6" t="inlineStr">
         <is>
           <t>Sección sin datos</t>
         </is>
       </c>
-      <c r="H78" s="6" t="inlineStr">
+      <c r="H79" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario aún no define su objetivo, no tiene citas o una sección todavía no existe</t>
         </is>
       </c>
-      <c r="I78" s="6" t="inlineStr">
+      <c r="I79" s="6" t="inlineStr">
         <is>
           <t>cuando abre el Inicio o esa sección</t>
         </is>
       </c>
-      <c r="J78" s="6" t="inlineStr">
+      <c r="J79" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra un estado vacío o el aviso "Próximamente" con la acción que corresponde, sin datos inventados</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="55" customHeight="1">
-      <c r="B79" s="20" t="n"/>
-      <c r="C79" s="20" t="n"/>
-      <c r="D79" s="20" t="n"/>
-      <c r="E79" s="20" t="n"/>
-      <c r="F79" s="8" t="n">
+    <row r="80" ht="55" customHeight="1">
+      <c r="B80" s="20" t="n"/>
+      <c r="C80" s="20" t="n"/>
+      <c r="D80" s="20" t="n"/>
+      <c r="E80" s="20" t="n"/>
+      <c r="F80" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G79" s="6" t="inlineStr">
+      <c r="G80" s="6" t="inlineStr">
         <is>
           <t>Menú de la cuenta</t>
         </is>
       </c>
-      <c r="H79" s="6" t="inlineStr">
+      <c r="H80" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario tiene la sesión iniciada</t>
         </is>
       </c>
-      <c r="I79" s="6" t="inlineStr">
+      <c r="I80" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Hola, {nombre}" o su avatar</t>
         </is>
       </c>
-      <c r="J79" s="6" t="inlineStr">
+      <c r="J80" s="6" t="inlineStr">
         <is>
           <t>el sistema abre un menú con "Mi perfil" y "Cerrar sesión"; cerrar sesión vuelve a la portada</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="55" customHeight="1"/>
-    <row r="81" ht="55" customHeight="1">
-      <c r="B81" s="6" t="inlineStr">
+    <row r="81" ht="55" customHeight="1"/>
+    <row r="82" ht="55" customHeight="1">
+      <c r="B82" s="6" t="inlineStr">
         <is>
           <t>FS-HU-22</t>
         </is>
       </c>
-      <c r="C81" s="6" t="inlineStr">
+      <c r="C82" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D81" s="6" t="inlineStr">
+      <c r="D82" s="6" t="inlineStr">
         <is>
           <t>Necesito buscar profesionales por texto y filtrarlos por especialidad, comuna, distancia, calificación y modalidad</t>
         </is>
       </c>
-      <c r="E81" s="6" t="inlineStr">
+      <c r="E82" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de encontrar rápidamente al profesional que se ajusta a lo que busco</t>
         </is>
       </c>
-      <c r="F81" s="8" t="n">
+      <c r="F82" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G81" s="6" t="inlineStr">
+      <c r="G82" s="6" t="inlineStr">
         <is>
           <t>Búsqueda con filtros</t>
         </is>
       </c>
-      <c r="H81" s="6" t="inlineStr">
+      <c r="H82" s="6" t="inlineStr">
         <is>
           <t>En caso que existen profesionales registrados</t>
         </is>
       </c>
-      <c r="I81" s="6" t="inlineStr">
+      <c r="I82" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario busca un texto y elige especialidad, comuna, calificación mínima o modalidad</t>
         </is>
       </c>
-      <c r="J81" s="6" t="inlineStr">
+      <c r="J82" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra solo los profesionales que cumplen los filtros, el total encontrado y el orden elegido</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="55" customHeight="1">
-      <c r="B82" s="22" t="n"/>
-      <c r="C82" s="22" t="n"/>
-      <c r="D82" s="22" t="n"/>
-      <c r="E82" s="22" t="n"/>
-      <c r="F82" s="8" t="n">
+    <row r="83" ht="55" customHeight="1">
+      <c r="B83" s="22" t="n"/>
+      <c r="C83" s="22" t="n"/>
+      <c r="D83" s="22" t="n"/>
+      <c r="E83" s="22" t="n"/>
+      <c r="F83" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G82" s="6" t="inlineStr">
+      <c r="G83" s="6" t="inlineStr">
         <is>
           <t>Búsqueda compartida</t>
         </is>
       </c>
-      <c r="H82" s="6" t="inlineStr">
+      <c r="H83" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario copia la dirección de una búsqueda</t>
         </is>
       </c>
-      <c r="I82" s="6" t="inlineStr">
+      <c r="I83" s="6" t="inlineStr">
         <is>
           <t>cuando otra persona con sesión la abre</t>
         </is>
       </c>
-      <c r="J82" s="6" t="inlineStr">
+      <c r="J83" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra la misma búsqueda con sus filtros, porque quedan guardados en la dirección (nunca la ubicación de la persona)</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="55" customHeight="1">
-      <c r="B83" s="20" t="n"/>
-      <c r="C83" s="20" t="n"/>
-      <c r="D83" s="20" t="n"/>
-      <c r="E83" s="20" t="n"/>
-      <c r="F83" s="8" t="n">
+    <row r="84" ht="55" customHeight="1">
+      <c r="B84" s="20" t="n"/>
+      <c r="C84" s="20" t="n"/>
+      <c r="D84" s="20" t="n"/>
+      <c r="E84" s="20" t="n"/>
+      <c r="F84" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G83" s="6" t="inlineStr">
+      <c r="G84" s="6" t="inlineStr">
         <is>
           <t>Sin coincidencias</t>
         </is>
       </c>
-      <c r="H83" s="6" t="inlineStr">
+      <c r="H84" s="6" t="inlineStr">
         <is>
           <t>En caso que ningún profesional cumple los filtros</t>
         </is>
       </c>
-      <c r="I83" s="6" t="inlineStr">
+      <c r="I84" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario aplica la búsqueda</t>
         </is>
       </c>
-      <c r="J83" s="6" t="inlineStr">
+      <c r="J84" s="6" t="inlineStr">
         <is>
           <t>el sistema indica "No encontramos profesionales con esos filtros" y ofrece limpiar los filtros</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="55" customHeight="1"/>
-    <row r="85" ht="55" customHeight="1">
-      <c r="B85" s="6" t="inlineStr">
+    <row r="85" ht="55" customHeight="1"/>
+    <row r="86" ht="55" customHeight="1">
+      <c r="B86" s="6" t="inlineStr">
         <is>
           <t>FS-HU-23</t>
         </is>
       </c>
-      <c r="C85" s="6" t="inlineStr">
+      <c r="C86" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D85" s="6" t="inlineStr">
+      <c r="D86" s="6" t="inlineStr">
         <is>
           <t>Necesito guardar profesionales como favoritos</t>
         </is>
       </c>
-      <c r="E85" s="6" t="inlineStr">
+      <c r="E86" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de volver a encontrarlos fácilmente</t>
         </is>
       </c>
-      <c r="F85" s="8" t="n">
+      <c r="F86" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G85" s="6" t="inlineStr">
+      <c r="G86" s="6" t="inlineStr">
         <is>
           <t>Guardar un favorito</t>
         </is>
       </c>
-      <c r="H85" s="6" t="inlineStr">
+      <c r="H86" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ve un profesional en el Inicio, el buscador o su ficha</t>
         </is>
       </c>
-      <c r="I85" s="6" t="inlineStr">
+      <c r="I86" s="6" t="inlineStr">
         <is>
           <t>cuando presiona el corazón</t>
         </is>
       </c>
-      <c r="J85" s="6" t="inlineStr">
+      <c r="J86" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda el profesional en sus favoritos y el corazón queda marcado</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="55" customHeight="1">
-      <c r="B86" s="22" t="n"/>
-      <c r="C86" s="22" t="n"/>
-      <c r="D86" s="22" t="n"/>
-      <c r="E86" s="22" t="n"/>
-      <c r="F86" s="8" t="n">
+    <row r="87" ht="55" customHeight="1">
+      <c r="B87" s="22" t="n"/>
+      <c r="C87" s="22" t="n"/>
+      <c r="D87" s="22" t="n"/>
+      <c r="E87" s="22" t="n"/>
+      <c r="F87" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G86" s="6" t="inlineStr">
+      <c r="G87" s="6" t="inlineStr">
         <is>
           <t>Ver favoritos</t>
         </is>
       </c>
-      <c r="H86" s="6" t="inlineStr">
+      <c r="H87" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario guardó profesionales</t>
         </is>
       </c>
-      <c r="I86" s="6" t="inlineStr">
+      <c r="I87" s="6" t="inlineStr">
         <is>
           <t>cuando abre "Favoritos" en el menú</t>
         </is>
       </c>
-      <c r="J86" s="6" t="inlineStr">
+      <c r="J87" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra sus profesionales guardados; si no tiene ninguno, explica cómo guardarlos</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="55" customHeight="1">
-      <c r="B87" s="20" t="n"/>
-      <c r="C87" s="20" t="n"/>
-      <c r="D87" s="20" t="n"/>
-      <c r="E87" s="20" t="n"/>
-      <c r="F87" s="8" t="n">
+    <row r="88" ht="55" customHeight="1">
+      <c r="B88" s="20" t="n"/>
+      <c r="C88" s="20" t="n"/>
+      <c r="D88" s="20" t="n"/>
+      <c r="E88" s="20" t="n"/>
+      <c r="F88" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G87" s="6" t="inlineStr">
+      <c r="G88" s="6" t="inlineStr">
         <is>
           <t>Quitar un favorito</t>
         </is>
       </c>
-      <c r="H87" s="6" t="inlineStr">
+      <c r="H88" s="6" t="inlineStr">
         <is>
           <t>En caso que un profesional está en favoritos</t>
         </is>
       </c>
-      <c r="I87" s="6" t="inlineStr">
+      <c r="I88" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario vuelve a presionar el corazón</t>
         </is>
       </c>
-      <c r="J87" s="6" t="inlineStr">
+      <c r="J88" s="6" t="inlineStr">
         <is>
           <t>el sistema lo quita de sus favoritos</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="55" customHeight="1"/>
-    <row r="89" ht="55" customHeight="1">
-      <c r="B89" s="6" t="inlineStr">
+    <row r="89" ht="55" customHeight="1"/>
+    <row r="90" ht="55" customHeight="1">
+      <c r="B90" s="6" t="inlineStr">
         <is>
           <t>FS-HU-24</t>
         </is>
       </c>
-      <c r="C89" s="6" t="inlineStr">
+      <c r="C90" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D89" s="6" t="inlineStr">
+      <c r="D90" s="6" t="inlineStr">
         <is>
           <t>Necesito calificar con estrellas a un profesional y comentar mi experiencia</t>
         </is>
       </c>
-      <c r="E89" s="6" t="inlineStr">
+      <c r="E90" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de ayudar a otras personas a elegir y conocer la opinión de quienes ya se atendieron</t>
         </is>
       </c>
-      <c r="F89" s="8" t="n">
+      <c r="F90" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G89" s="6" t="inlineStr">
+      <c r="G90" s="6" t="inlineStr">
         <is>
           <t>Publicar una reseña</t>
         </is>
       </c>
-      <c r="H89" s="6" t="inlineStr">
+      <c r="H90" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario abre la ficha de un profesional</t>
         </is>
       </c>
-      <c r="I89" s="6" t="inlineStr">
+      <c r="I90" s="6" t="inlineStr">
         <is>
           <t>cuando elige de 1 a 5 estrellas y, si quiere, escribe un comentario de 10 a 500 caracteres</t>
         </is>
       </c>
-      <c r="J89" s="6" t="inlineStr">
+      <c r="J90" s="6" t="inlineStr">
         <is>
           <t>el sistema publica la reseña con su nombre abreviado y actualiza el promedio y la cantidad de reseñas</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="55" customHeight="1">
-      <c r="B90" s="22" t="n"/>
-      <c r="C90" s="22" t="n"/>
-      <c r="D90" s="22" t="n"/>
-      <c r="E90" s="22" t="n"/>
-      <c r="F90" s="8" t="n">
+    <row r="91" ht="55" customHeight="1">
+      <c r="B91" s="22" t="n"/>
+      <c r="C91" s="22" t="n"/>
+      <c r="D91" s="22" t="n"/>
+      <c r="E91" s="22" t="n"/>
+      <c r="F91" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G90" s="6" t="inlineStr">
+      <c r="G91" s="6" t="inlineStr">
         <is>
           <t>Editar o eliminar su reseña</t>
         </is>
       </c>
-      <c r="H90" s="6" t="inlineStr">
+      <c r="H91" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ya calificó a ese profesional</t>
         </is>
       </c>
-      <c r="I90" s="6" t="inlineStr">
+      <c r="I91" s="6" t="inlineStr">
         <is>
           <t>cuando edita o elimina su reseña</t>
         </is>
       </c>
-      <c r="J90" s="6" t="inlineStr">
+      <c r="J91" s="6" t="inlineStr">
         <is>
           <t>el sistema reemplaza o elimina su única reseña y recalcula el promedio</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="55" customHeight="1">
-      <c r="B91" s="20" t="n"/>
-      <c r="C91" s="20" t="n"/>
-      <c r="D91" s="20" t="n"/>
-      <c r="E91" s="20" t="n"/>
-      <c r="F91" s="8" t="n">
+    <row r="92" ht="55" customHeight="1">
+      <c r="B92" s="20" t="n"/>
+      <c r="C92" s="20" t="n"/>
+      <c r="D92" s="20" t="n"/>
+      <c r="E92" s="20" t="n"/>
+      <c r="F92" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G91" s="6" t="inlineStr">
+      <c r="G92" s="6" t="inlineStr">
         <is>
           <t>Cuenta que no puede calificar</t>
         </is>
       </c>
-      <c r="H91" s="6" t="inlineStr">
+      <c r="H92" s="6" t="inlineStr">
         <is>
           <t>En caso que una cuenta profesional abre una ficha (o la suya propia)</t>
         </is>
       </c>
-      <c r="I91" s="6" t="inlineStr">
+      <c r="I92" s="6" t="inlineStr">
         <is>
           <t>cuando intenta calificar</t>
         </is>
       </c>
-      <c r="J91" s="6" t="inlineStr">
+      <c r="J92" s="6" t="inlineStr">
         <is>
           <t>el sistema le permite leer las reseñas, pero no calificar, y rechaza la calificación si se envía igual</t>
         </is>
       </c>
     </row>
-    <row r="92"/>
-    <row r="93">
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Nota:</t>
-        </is>
-      </c>
-    </row>
+    <row r="93"/>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>- Se utilizaron 2 escenarios (criterios de aceptación) por historia de usuario: el caso principal (camino feliz) y un caso de error o borde relevante; FS-HU-14 incluye un tercer escenario para confirmar o cancelar la reserva; FS-HU-15 a FS-HU-24 también incluyen tres escenarios.</t>
+          <t>Nota:</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
+          <t>- Se utilizaron 2 escenarios (criterios de aceptación) por historia de usuario: el caso principal (camino feliz) y un caso de error o borde relevante; FS-HU-14 incluye un tercer escenario para confirmar o cancelar la reserva; FS-HU-15 a FS-HU-24 también incluyen tres escenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" t="inlineStr">
+        <is>
           <t>- El detalle completo de las 24 historias también está disponible en el Product Backlog (PMOInformatica_Plantilla_de_Product_Backlog.xlsx).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="98">
-    <mergeCell ref="B53:B55"/>
-    <mergeCell ref="D53:D55"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="C61:C63"/>
+    <mergeCell ref="B43:B44"/>
     <mergeCell ref="G4:J4"/>
-    <mergeCell ref="D25:D27"/>
-    <mergeCell ref="B42:B43"/>
     <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="C81:C83"/>
-    <mergeCell ref="D45:D46"/>
+    <mergeCell ref="E26:E28"/>
     <mergeCell ref="D9:D11"/>
-    <mergeCell ref="E48:E51"/>
+    <mergeCell ref="D30:D32"/>
+    <mergeCell ref="C78:C80"/>
     <mergeCell ref="B13:B14"/>
-    <mergeCell ref="E81:E83"/>
     <mergeCell ref="D13:D14"/>
-    <mergeCell ref="D48:D51"/>
-    <mergeCell ref="D29:D31"/>
     <mergeCell ref="D16:D17"/>
     <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C89:C91"/>
-    <mergeCell ref="D65:D67"/>
-    <mergeCell ref="C73:C75"/>
-    <mergeCell ref="E73:E75"/>
-    <mergeCell ref="B57:B59"/>
-    <mergeCell ref="D57:D59"/>
-    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="C58:C60"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="E58:E60"/>
+    <mergeCell ref="D22:D24"/>
+    <mergeCell ref="B62:B64"/>
+    <mergeCell ref="C43:C44"/>
+    <mergeCell ref="E82:E84"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="B70:B72"/>
+    <mergeCell ref="D70:D72"/>
+    <mergeCell ref="D34:D35"/>
     <mergeCell ref="C6:C7"/>
-    <mergeCell ref="E61:E63"/>
-    <mergeCell ref="E77:E79"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="C49:C52"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="E30:E32"/>
     <mergeCell ref="E13:E14"/>
-    <mergeCell ref="C45:C46"/>
-    <mergeCell ref="C69:C71"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="B85:B87"/>
-    <mergeCell ref="D85:D87"/>
-    <mergeCell ref="D69:D71"/>
+    <mergeCell ref="E86:E88"/>
+    <mergeCell ref="D49:D52"/>
+    <mergeCell ref="B74:B76"/>
+    <mergeCell ref="E22:E24"/>
+    <mergeCell ref="E62:E64"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="C62:C64"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="C54:C56"/>
     <mergeCell ref="C4:F4"/>
-    <mergeCell ref="D61:D63"/>
-    <mergeCell ref="B45:B46"/>
-    <mergeCell ref="C48:C51"/>
-    <mergeCell ref="D39:D40"/>
+    <mergeCell ref="D37:D38"/>
     <mergeCell ref="C19:C20"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="C26:C28"/>
+    <mergeCell ref="D86:D88"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="C90:C92"/>
+    <mergeCell ref="E90:E92"/>
     <mergeCell ref="B16:B17"/>
-    <mergeCell ref="E65:E67"/>
     <mergeCell ref="C9:C11"/>
     <mergeCell ref="E9:E11"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="B65:B67"/>
-    <mergeCell ref="E42:E43"/>
-    <mergeCell ref="E85:E87"/>
-    <mergeCell ref="B89:B91"/>
-    <mergeCell ref="D89:D91"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="C53:C55"/>
-    <mergeCell ref="E53:E55"/>
-    <mergeCell ref="D73:D75"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="C29:C31"/>
-    <mergeCell ref="E29:E31"/>
-    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="E74:E76"/>
+    <mergeCell ref="B78:B80"/>
+    <mergeCell ref="D78:D80"/>
+    <mergeCell ref="D74:D76"/>
+    <mergeCell ref="C82:C84"/>
+    <mergeCell ref="D58:D60"/>
+    <mergeCell ref="C66:C68"/>
+    <mergeCell ref="E66:E68"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="D26:D28"/>
+    <mergeCell ref="B66:B68"/>
+    <mergeCell ref="D82:D84"/>
+    <mergeCell ref="C86:C88"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C30:C32"/>
+    <mergeCell ref="D43:D44"/>
     <mergeCell ref="E16:E17"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="B77:B79"/>
-    <mergeCell ref="D77:D79"/>
-    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B49:B52"/>
+    <mergeCell ref="E78:E80"/>
+    <mergeCell ref="B86:B88"/>
     <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E89:E91"/>
-    <mergeCell ref="C57:C59"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="E57:E59"/>
-    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="D62:D64"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="C70:C72"/>
+    <mergeCell ref="E70:E72"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="E54:E56"/>
+    <mergeCell ref="D46:D47"/>
     <mergeCell ref="E19:E20"/>
-    <mergeCell ref="C77:C79"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="E25:E27"/>
+    <mergeCell ref="E34:E35"/>
+    <mergeCell ref="B54:B56"/>
+    <mergeCell ref="D54:D56"/>
     <mergeCell ref="E6:E7"/>
     <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B48:B51"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="B81:B83"/>
-    <mergeCell ref="D81:D83"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="C85:C87"/>
+    <mergeCell ref="E49:E52"/>
+    <mergeCell ref="C74:C76"/>
+    <mergeCell ref="B90:B92"/>
+    <mergeCell ref="D90:D92"/>
+    <mergeCell ref="B58:B60"/>
     <mergeCell ref="C13:C14"/>
     <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E69:E71"/>
-    <mergeCell ref="C65:C67"/>
-    <mergeCell ref="B73:B75"/>
-    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="B82:B84"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="E37:E38"/>
     <mergeCell ref="B9:B11"/>
-    <mergeCell ref="B69:B71"/>
-    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="D66:D68"/>
   </mergeCells>
   <pageMargins left="0.7086614173228347" right="0.7086614173228347" top="0.7480314960629921" bottom="0.7480314960629921" header="0.3149606299212598" footer="0.3149606299212598"/>
   <pageSetup orientation="landscape" paperSize="9" scale="70"/>

</xml_diff>

<commit_message>
Documentacion del modulo Comidas: DAS 1.29, diagramas 02, 03, 04, 07, 08 y 15, escenarios de FS-HU-09 y FS-HU-10 y README
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Material complementario/Plantilla_Historias_Usuario_con_instructivo.xlsx
+++ b/FASE 1/Evidencias Grupales/Material complementario/Plantilla_Historias_Usuario_con_instructivo.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J97"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
     <col width="1.44140625" customWidth="1" style="5" min="1" max="1"/>
@@ -1524,22 +1524,22 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>Registro de una comida completa</t>
+          <t>Agregar alimentos desde el chat</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>En caso que el usuario describe una comida en lenguaje natural (ej. "2 huevos y un plátano")</t>
+          <t>En caso que el usuario le pide al asistente agregar lo que comió (ej. «agrega 100 g de pollo y 150 g de arroz a mi almuerzo»)</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>cuando confirma el registro sugerido por el asistente</t>
+          <t>cuando envía el mensaje</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
-          <t>el sistema guarda los alimentos, cantidades y la estimación nutricional en el gestor de alimentación</t>
+          <t>el sistema busca cada alimento en el catálogo, lo registra con sus gramos y su aporte nutricional en las comidas de hoy (en el momento indicado o según la hora) y muestra lo agregado con acceso a Comidas</t>
         </is>
       </c>
     </row>
@@ -1558,17 +1558,17 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>En caso que el usuario menciona un alimento que el sistema no logra identificar</t>
+          <t>En caso que el usuario menciona un alimento que no está en el catálogo o una cantidad no válida</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>cuando confirma igualmente el registro</t>
+          <t>cuando pide agregarlo</t>
         </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>el sistema guarda el resto de los alimentos reconocidos y señala cuál no pudo identificar</t>
+          <t>el sistema agrega solo los alimentos reconocidos y le indica cuál no pudo registrar, para que lo registre en Comidas eligiendo uno parecido</t>
         </is>
       </c>
     </row>
@@ -1599,351 +1599,351 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Consulta de progreso diario</t>
+          <t>Registrar un alimento con sus gramos</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>En caso que el usuario ya registró comidas durante el día</t>
+          <t>En caso que el usuario busca un alimento del catálogo en Comidas</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>cuando abre el resumen de calorías y macronutrientes</t>
+          <t>cuando indica el momento del día y los gramos y lo agrega</t>
         </is>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>el sistema muestra el consumo del día comparado con su objetivo diario</t>
+          <t>el sistema calcula y guarda sus calorías y macronutrientes y actualiza el resumen del día</t>
         </is>
       </c>
     </row>
     <row r="38" ht="55" customHeight="1">
-      <c r="B38" s="20" t="n"/>
-      <c r="C38" s="20" t="n"/>
-      <c r="D38" s="20" t="n"/>
-      <c r="E38" s="20" t="n"/>
+      <c r="B38" s="22" t="n"/>
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="22" t="n"/>
+      <c r="E38" s="22" t="n"/>
       <c r="F38" s="8" t="n">
         <v>2</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>Sin registros en el día</t>
+          <t>Consulta de progreso diario</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>En caso que el usuario no ha registrado ninguna comida en el día</t>
+          <t>En caso que el usuario ya registró comidas durante el día</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>cuando abre el resumen de progreso</t>
+          <t>cuando abre el resumen de Comidas</t>
         </is>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>el sistema muestra el objetivo diario completo como pendiente, sin errores</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="55" customHeight="1"/>
-    <row r="40" ht="55" customHeight="1">
-      <c r="B40" s="6" t="inlineStr">
+          <t>el sistema muestra las calorías y macronutrientes consumidos frente a su objetivo diario (calculado con su perfil) y el progreso de la semana</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="55" customHeight="1">
+      <c r="B39" s="20" t="n"/>
+      <c r="C39" s="20" t="n"/>
+      <c r="D39" s="20" t="n"/>
+      <c r="E39" s="20" t="n"/>
+      <c r="F39" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>Sin registros o sin perfil completo</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>En caso que el usuario no ha registrado comidas en el día o no ha completado su perfil</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>cuando abre el resumen de Comidas</t>
+        </is>
+      </c>
+      <c r="J39" s="6" t="inlineStr">
+        <is>
+          <t>el sistema muestra el objetivo del día como pendiente, sin errores, o, si falta el perfil, el consumo sin objetivo y lo invita a completarlo</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="55" customHeight="1"/>
+    <row r="41" ht="55" customHeight="1">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>FS-HU-11</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>Como un equipo de desarrollo</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Necesito dockerizar la aplicación completa</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de que cualquiera pueda instalarla y ejecutarla fácilmente</t>
         </is>
       </c>
-      <c r="F40" s="8" t="n">
+      <c r="F41" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G40" s="6" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>Levantar el entorno completo</t>
         </is>
       </c>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>En caso que un desarrollador clona el repositorio por primera vez</t>
         </is>
       </c>
-      <c r="I40" s="6" t="inlineStr">
+      <c r="I41" s="6" t="inlineStr">
         <is>
           <t>cuando ejecuta docker-compose up</t>
         </is>
       </c>
-      <c r="J40" s="6" t="inlineStr">
+      <c r="J41" s="6" t="inlineStr">
         <is>
           <t>el sistema levanta frontend, backend y base de datos MySQL correctamente configurados</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="55" customHeight="1">
-      <c r="B41" s="20" t="n"/>
-      <c r="C41" s="20" t="n"/>
-      <c r="D41" s="20" t="n"/>
-      <c r="E41" s="20" t="n"/>
-      <c r="F41" s="8" t="n">
+    <row r="42" ht="55" customHeight="1">
+      <c r="B42" s="20" t="n"/>
+      <c r="C42" s="20" t="n"/>
+      <c r="D42" s="20" t="n"/>
+      <c r="E42" s="20" t="n"/>
+      <c r="F42" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G41" s="6" t="inlineStr">
+      <c r="G42" s="6" t="inlineStr">
         <is>
           <t>Variables de entorno faltantes</t>
         </is>
       </c>
-      <c r="H41" s="6" t="inlineStr">
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>En caso que el archivo de variables de entorno no está configurado</t>
         </is>
       </c>
-      <c r="I41" s="6" t="inlineStr">
+      <c r="I42" s="6" t="inlineStr">
         <is>
           <t>cuando se intenta levantar el entorno</t>
         </is>
       </c>
-      <c r="J41" s="6" t="inlineStr">
+      <c r="J42" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra un error claro indicando qué variable falta</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="55" customHeight="1"/>
-    <row r="43" ht="55" customHeight="1">
-      <c r="B43" s="6" t="inlineStr">
+    <row r="43" ht="55" customHeight="1"/>
+    <row r="44" ht="55" customHeight="1">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>FS-HU-12</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>Como un administrador</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>Necesito verificar los perfiles de los profesionales</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de que los usuarios identifiquen a los profesionales validados por la plataforma</t>
         </is>
       </c>
-      <c r="F43" s="8" t="n">
+      <c r="F44" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G43" s="6" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
         <is>
           <t>Verificación de un perfil</t>
         </is>
       </c>
-      <c r="H43" s="6" t="inlineStr">
+      <c r="H44" s="6" t="inlineStr">
         <is>
           <t>En caso que existe un perfil profesional pendiente de verificación</t>
         </is>
       </c>
-      <c r="I43" s="6" t="inlineStr">
+      <c r="I44" s="6" t="inlineStr">
         <is>
           <t>cuando el administrador lo revisa y lo marca como verificado</t>
         </is>
       </c>
-      <c r="J43" s="6" t="inlineStr">
+      <c r="J44" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda el estado verificado y muestra una insignia de verificación en el perfil y en el listado de profesionales</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="55" customHeight="1">
-      <c r="B44" s="20" t="n"/>
-      <c r="C44" s="20" t="n"/>
-      <c r="D44" s="20" t="n"/>
-      <c r="E44" s="20" t="n"/>
-      <c r="F44" s="8" t="n">
+    <row r="45" ht="55" customHeight="1">
+      <c r="B45" s="20" t="n"/>
+      <c r="C45" s="20" t="n"/>
+      <c r="D45" s="20" t="n"/>
+      <c r="E45" s="20" t="n"/>
+      <c r="F45" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G44" s="6" t="inlineStr">
+      <c r="G45" s="6" t="inlineStr">
         <is>
           <t>Acceso no autorizado</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr">
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>En caso que un usuario sin rol de administrador intenta verificar un perfil</t>
         </is>
       </c>
-      <c r="I44" s="6" t="inlineStr">
+      <c r="I45" s="6" t="inlineStr">
         <is>
           <t>cuando envía la solicitud de verificación</t>
         </is>
       </c>
-      <c r="J44" s="6" t="inlineStr">
+      <c r="J45" s="6" t="inlineStr">
         <is>
           <t>el sistema rechaza la acción y no modifica el perfil</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="55" customHeight="1"/>
-    <row r="46" ht="55" customHeight="1">
-      <c r="B46" s="6" t="inlineStr">
+    <row r="46" ht="55" customHeight="1"/>
+    <row r="47" ht="55" customHeight="1">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>FS-HU-13</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Como un profesional</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Necesito definir mis horarios disponibles</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de que los usuarios puedan reservar una hora conmigo</t>
         </is>
       </c>
-      <c r="F46" s="8" t="n">
+      <c r="F47" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G46" s="6" t="inlineStr">
+      <c r="G47" s="6" t="inlineStr">
         <is>
           <t>Registrar bloques de disponibilidad</t>
         </is>
       </c>
-      <c r="H46" s="6" t="inlineStr">
+      <c r="H47" s="6" t="inlineStr">
         <is>
           <t>En caso que un profesional tiene su perfil creado</t>
         </is>
       </c>
-      <c r="I46" s="6" t="inlineStr">
+      <c r="I47" s="6" t="inlineStr">
         <is>
           <t>cuando agrega un bloque indicando fecha, hora de inicio y hora de término</t>
         </is>
       </c>
-      <c r="J46" s="6" t="inlineStr">
+      <c r="J47" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda el bloque y lo muestra como horario disponible en su perfil</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="55" customHeight="1">
-      <c r="B47" s="20" t="n"/>
-      <c r="C47" s="20" t="n"/>
-      <c r="D47" s="20" t="n"/>
-      <c r="E47" s="20" t="n"/>
-      <c r="F47" s="8" t="n">
+    <row r="48" ht="55" customHeight="1">
+      <c r="B48" s="20" t="n"/>
+      <c r="C48" s="20" t="n"/>
+      <c r="D48" s="20" t="n"/>
+      <c r="E48" s="20" t="n"/>
+      <c r="F48" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G47" s="6" t="inlineStr">
+      <c r="G48" s="6" t="inlineStr">
         <is>
           <t>Bloque inválido o superpuesto</t>
         </is>
       </c>
-      <c r="H47" s="6" t="inlineStr">
+      <c r="H48" s="6" t="inlineStr">
         <is>
           <t>En caso que el profesional ingresa un bloque cuya hora de término no es posterior a la de inicio o que se superpone con otro bloque</t>
         </is>
       </c>
-      <c r="I47" s="6" t="inlineStr">
+      <c r="I48" s="6" t="inlineStr">
         <is>
           <t>cuando intenta guardarlo</t>
         </is>
       </c>
-      <c r="J47" s="6" t="inlineStr">
+      <c r="J48" s="6" t="inlineStr">
         <is>
           <t>el sistema no guarda el bloque e indica el problema</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="55" customHeight="1"/>
-    <row r="49" ht="55" customHeight="1">
-      <c r="B49" s="6" t="inlineStr">
+    <row r="49" ht="55" customHeight="1"/>
+    <row r="50" ht="55" customHeight="1">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>FS-HU-14</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>Necesito reservar una hora con un profesional indicando brevemente lo que necesito</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de agendar una atención que se ajuste a mi necesidad</t>
         </is>
       </c>
-      <c r="F49" s="8" t="n">
+      <c r="F50" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G49" s="6" t="inlineStr">
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t>Reserva con mensaje</t>
         </is>
       </c>
-      <c r="H49" s="6" t="inlineStr">
+      <c r="H50" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ve un horario disponible en el perfil de un profesional</t>
         </is>
       </c>
-      <c r="I49" s="6" t="inlineStr">
+      <c r="I50" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Reservar", escribe un mensaje breve con lo que necesita y confirma</t>
         </is>
       </c>
-      <c r="J49" s="6" t="inlineStr">
+      <c r="J50" s="6" t="inlineStr">
         <is>
           <t>el sistema crea la reserva en estado pendiente, el horario deja de estar disponible y el profesional ve la reserva junto al mensaje</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="55" customHeight="1">
-      <c r="B50" s="22" t="n"/>
-      <c r="C50" s="22" t="n"/>
-      <c r="D50" s="22" t="n"/>
-      <c r="E50" s="22" t="n"/>
-      <c r="F50" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>Reserva sin mensaje u horario ocupado</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr">
-        <is>
-          <t>En caso que el usuario no escribe el mensaje o el horario fue tomado por otro usuario</t>
-        </is>
-      </c>
-      <c r="I50" s="6" t="inlineStr">
-        <is>
-          <t>cuando intenta confirmar la reserva</t>
-        </is>
-      </c>
-      <c r="J50" s="6" t="inlineStr">
-        <is>
-          <t>el sistema no crea la reserva e indica que debe escribir el mensaje o elegir otro horario</t>
         </is>
       </c>
     </row>
@@ -1953,1222 +1953,1251 @@
       <c r="D51" s="22" t="n"/>
       <c r="E51" s="22" t="n"/>
       <c r="F51" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Reserva sin mensaje u horario ocupado</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>En caso que el usuario no escribe el mensaje o el horario fue tomado por otro usuario</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>cuando intenta confirmar la reserva</t>
+        </is>
+      </c>
+      <c r="J51" s="6" t="inlineStr">
+        <is>
+          <t>el sistema no crea la reserva e indica que debe escribir el mensaje o elegir otro horario</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="55" customHeight="1">
+      <c r="B52" s="22" t="n"/>
+      <c r="C52" s="22" t="n"/>
+      <c r="D52" s="22" t="n"/>
+      <c r="E52" s="22" t="n"/>
+      <c r="F52" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G51" s="6" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>Confirmar o cancelar una reserva</t>
         </is>
       </c>
-      <c r="H51" s="6" t="inlineStr">
+      <c r="H52" s="6" t="inlineStr">
         <is>
           <t>En caso que existe una reserva pendiente</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr">
+      <c r="I52" s="6" t="inlineStr">
         <is>
           <t>cuando el profesional la confirma o cualquiera de las partes la cancela</t>
         </is>
       </c>
-      <c r="J51" s="6" t="inlineStr">
+      <c r="J52" s="6" t="inlineStr">
         <is>
           <t>el sistema actualiza el estado, libera el horario si se cancela y ambas partes ven el estado actualizado</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="55" customHeight="1">
-      <c r="B52" s="20" t="n"/>
-      <c r="C52" s="20" t="n"/>
-      <c r="D52" s="20" t="n"/>
-      <c r="E52" s="20" t="n"/>
-      <c r="F52" s="8" t="inlineStr">
+    <row r="53" ht="55" customHeight="1">
+      <c r="B53" s="20" t="n"/>
+      <c r="C53" s="20" t="n"/>
+      <c r="D53" s="20" t="n"/>
+      <c r="E53" s="20" t="n"/>
+      <c r="F53" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G52" s="6" t="inlineStr">
+      <c r="G53" s="6" t="inlineStr">
         <is>
           <t>Límite de una reserva activa por profesional</t>
         </is>
       </c>
-      <c r="H52" s="6" t="inlineStr">
+      <c r="H53" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ya tiene una reserva pendiente o confirmada para un horario futuro con ese profesional</t>
         </is>
       </c>
-      <c r="I52" s="6" t="inlineStr">
+      <c r="I53" s="6" t="inlineStr">
         <is>
           <t>cuando intenta reservar otra hora con el mismo profesional</t>
         </is>
       </c>
-      <c r="J52" s="6" t="inlineStr">
+      <c r="J53" s="6" t="inlineStr">
         <is>
           <t>el sistema no crea la reserva, se lo avisa antes de escribir el mensaje y le indica que primero cancele la reserva activa en "Mis citas"; las citas que ya pasaron no cuentan para este límite (decisión del Product Owner del 12-10-2026)</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="55" customHeight="1"/>
-    <row r="54" ht="55" customHeight="1">
-      <c r="B54" s="6" t="inlineStr">
+    <row r="54" ht="55" customHeight="1"/>
+    <row r="55" ht="55" customHeight="1">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>FS-HU-15</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>Necesito recuperar mi contraseña mediante un enlace enviado a mi correo</t>
         </is>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de volver a acceder a mi cuenta si la olvido</t>
         </is>
       </c>
-      <c r="F54" s="8" t="n">
+      <c r="F55" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G54" s="6" t="inlineStr">
+      <c r="G55" s="6" t="inlineStr">
         <is>
           <t>Solicitar enlace de recuperación</t>
         </is>
       </c>
-      <c r="H54" s="6" t="inlineStr">
+      <c r="H55" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario olvidó su contraseña</t>
         </is>
       </c>
-      <c r="I54" s="6" t="inlineStr">
+      <c r="I55" s="6" t="inlineStr">
         <is>
           <t>cuando escribe su correo en "¿Olvidaste tu contraseña?" y presiona "Enviar enlace"</t>
         </is>
       </c>
-      <c r="J54" s="6" t="inlineStr">
+      <c r="J55" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra siempre el mismo mensaje de confirmación y, si el correo está registrado, envía un correo con un enlace válido por 60 minutos</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="55" customHeight="1">
-      <c r="B55" s="22" t="n"/>
-      <c r="C55" s="22" t="n"/>
-      <c r="D55" s="22" t="n"/>
-      <c r="E55" s="22" t="n"/>
-      <c r="F55" s="8" t="n">
+    <row r="56" ht="55" customHeight="1">
+      <c r="B56" s="22" t="n"/>
+      <c r="C56" s="22" t="n"/>
+      <c r="D56" s="22" t="n"/>
+      <c r="E56" s="22" t="n"/>
+      <c r="F56" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G55" s="6" t="inlineStr">
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>Restablecer la contraseña</t>
         </is>
       </c>
-      <c r="H55" s="6" t="inlineStr">
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario abre un enlace de recuperación vigente</t>
         </is>
       </c>
-      <c r="I55" s="6" t="inlineStr">
+      <c r="I56" s="6" t="inlineStr">
         <is>
           <t>cuando escribe una contraseña nueva de al menos 8 caracteres y su confirmación coincide</t>
         </is>
       </c>
-      <c r="J55" s="6" t="inlineStr">
+      <c r="J56" s="6" t="inlineStr">
         <is>
           <t>el sistema actualiza la contraseña, inutiliza el enlace y permite iniciar sesión con la contraseña nueva</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="55" customHeight="1">
-      <c r="B56" s="20" t="n"/>
-      <c r="C56" s="20" t="n"/>
-      <c r="D56" s="20" t="n"/>
-      <c r="E56" s="20" t="n"/>
-      <c r="F56" s="8" t="n">
+    <row r="57" ht="55" customHeight="1">
+      <c r="B57" s="20" t="n"/>
+      <c r="C57" s="20" t="n"/>
+      <c r="D57" s="20" t="n"/>
+      <c r="E57" s="20" t="n"/>
+      <c r="F57" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G56" s="6" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>Enlace vencido o usado</t>
         </is>
       </c>
-      <c r="H56" s="6" t="inlineStr">
+      <c r="H57" s="6" t="inlineStr">
         <is>
           <t>En caso que el enlace ya venció, ya se usó o fue alterado</t>
         </is>
       </c>
-      <c r="I56" s="6" t="inlineStr">
+      <c r="I57" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario intenta restablecer la contraseña</t>
         </is>
       </c>
-      <c r="J56" s="6" t="inlineStr">
+      <c r="J57" s="6" t="inlineStr">
         <is>
           <t>el sistema no cambia la contraseña e indica que debe solicitar un enlace nuevo</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="55" customHeight="1"/>
-    <row r="58" ht="55" customHeight="1">
-      <c r="B58" s="6" t="inlineStr">
+    <row r="58" ht="55" customHeight="1"/>
+    <row r="59" ht="55" customHeight="1">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>FS-HU-16</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>Como un usuario o profesional</t>
         </is>
       </c>
-      <c r="D58" s="6" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>Necesito registrarme e iniciar sesión con mi cuenta de Google</t>
         </is>
       </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de acceder sin crear ni recordar otra contraseña</t>
         </is>
       </c>
-      <c r="F58" s="8" t="n">
+      <c r="F59" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G58" s="6" t="inlineStr">
+      <c r="G59" s="6" t="inlineStr">
         <is>
           <t>Primer acceso con Google</t>
         </is>
       </c>
-      <c r="H58" s="6" t="inlineStr">
+      <c r="H59" s="6" t="inlineStr">
         <is>
           <t>En caso que la persona no tiene cuenta en FitSearch</t>
         </is>
       </c>
-      <c r="I58" s="6" t="inlineStr">
+      <c r="I59" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Continuar con Google" y autoriza el acceso</t>
         </is>
       </c>
-      <c r="J58" s="6" t="inlineStr">
+      <c r="J59" s="6" t="inlineStr">
         <is>
           <t>el sistema crea la cuenta y su perfil vacío, deja la sesión iniciada y le pide elegir su tipo de cuenta en el primer paso del perfil</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="55" customHeight="1">
-      <c r="B59" s="22" t="n"/>
-      <c r="C59" s="22" t="n"/>
-      <c r="D59" s="22" t="n"/>
-      <c r="E59" s="22" t="n"/>
-      <c r="F59" s="8" t="n">
+    <row r="60" ht="55" customHeight="1">
+      <c r="B60" s="22" t="n"/>
+      <c r="C60" s="22" t="n"/>
+      <c r="D60" s="22" t="n"/>
+      <c r="E60" s="22" t="n"/>
+      <c r="F60" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G59" s="6" t="inlineStr">
+      <c r="G60" s="6" t="inlineStr">
         <is>
           <t>Cuenta existente con el mismo correo</t>
         </is>
       </c>
-      <c r="H59" s="6" t="inlineStr">
+      <c r="H60" s="6" t="inlineStr">
         <is>
           <t>En caso que ya existe una cuenta registrada con el correo de Google</t>
         </is>
       </c>
-      <c r="I59" s="6" t="inlineStr">
+      <c r="I60" s="6" t="inlineStr">
         <is>
           <t>cuando la persona continúa con Google</t>
         </is>
       </c>
-      <c r="J59" s="6" t="inlineStr">
+      <c r="J60" s="6" t="inlineStr">
         <is>
           <t>el sistema vincula la cuenta de Google a la cuenta existente e inicia la sesión sin crear un usuario duplicado</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="55" customHeight="1">
-      <c r="B60" s="20" t="n"/>
-      <c r="C60" s="20" t="n"/>
-      <c r="D60" s="20" t="n"/>
-      <c r="E60" s="20" t="n"/>
-      <c r="F60" s="8" t="n">
+    <row r="61" ht="55" customHeight="1">
+      <c r="B61" s="20" t="n"/>
+      <c r="C61" s="20" t="n"/>
+      <c r="D61" s="20" t="n"/>
+      <c r="E61" s="20" t="n"/>
+      <c r="F61" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G60" s="6" t="inlineStr">
+      <c r="G61" s="6" t="inlineStr">
         <is>
           <t>Acceso con Google inválido</t>
         </is>
       </c>
-      <c r="H60" s="6" t="inlineStr">
+      <c r="H61" s="6" t="inlineStr">
         <is>
           <t>En caso que la validación de Google falla o el correo no está verificado</t>
         </is>
       </c>
-      <c r="I60" s="6" t="inlineStr">
+      <c r="I61" s="6" t="inlineStr">
         <is>
           <t>cuando el sistema recibe la solicitud de acceso</t>
         </is>
       </c>
-      <c r="J60" s="6" t="inlineStr">
+      <c r="J61" s="6" t="inlineStr">
         <is>
           <t>el sistema rechaza el acceso y muestra un mensaje de error sin crear la cuenta</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="55" customHeight="1"/>
-    <row r="62" ht="55" customHeight="1">
-      <c r="B62" s="6" t="inlineStr">
+    <row r="62" ht="55" customHeight="1"/>
+    <row r="63" ht="55" customHeight="1">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>FS-HU-17</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr">
+      <c r="C63" s="6" t="inlineStr">
         <is>
           <t>Como un usuario o profesional</t>
         </is>
       </c>
-      <c r="D62" s="6" t="inlineStr">
+      <c r="D63" s="6" t="inlineStr">
         <is>
           <t>Necesito confirmar mi contraseña al registrarme y decidir si mantener mi sesión iniciada</t>
         </is>
       </c>
-      <c r="E62" s="6" t="inlineStr">
+      <c r="E63" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de acceder a las funciones que me corresponden de forma cómoda y segura</t>
         </is>
       </c>
-      <c r="F62" s="8" t="n">
+      <c r="F63" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G62" s="6" t="inlineStr">
+      <c r="G63" s="6" t="inlineStr">
         <is>
           <t>Registro sin elegir rol</t>
         </is>
       </c>
-      <c r="H62" s="6" t="inlineStr">
+      <c r="H63" s="6" t="inlineStr">
         <is>
           <t>En caso que la persona completa el formulario de registro</t>
         </is>
       </c>
-      <c r="I62" s="6" t="inlineStr">
+      <c r="I63" s="6" t="inlineStr">
         <is>
           <t>cuando confirma el registro</t>
         </is>
       </c>
-      <c r="J62" s="6" t="inlineStr">
+      <c r="J63" s="6" t="inlineStr">
         <is>
           <t>el sistema crea la cuenta como usuario y le pide elegir su tipo de cuenta en el perfil; nunca permite registrarse como administrador</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="55" customHeight="1">
-      <c r="B63" s="22" t="n"/>
-      <c r="C63" s="22" t="n"/>
-      <c r="D63" s="22" t="n"/>
-      <c r="E63" s="22" t="n"/>
-      <c r="F63" s="8" t="n">
+    <row r="64" ht="55" customHeight="1">
+      <c r="B64" s="22" t="n"/>
+      <c r="C64" s="22" t="n"/>
+      <c r="D64" s="22" t="n"/>
+      <c r="E64" s="22" t="n"/>
+      <c r="F64" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G63" s="6" t="inlineStr">
+      <c r="G64" s="6" t="inlineStr">
         <is>
           <t>Contraseñas distintas</t>
         </is>
       </c>
-      <c r="H63" s="6" t="inlineStr">
+      <c r="H64" s="6" t="inlineStr">
         <is>
           <t>En caso que la contraseña y su confirmación no coinciden</t>
         </is>
       </c>
-      <c r="I63" s="6" t="inlineStr">
+      <c r="I64" s="6" t="inlineStr">
         <is>
           <t>cuando la persona intenta registrarse</t>
         </is>
       </c>
-      <c r="J63" s="6" t="inlineStr">
+      <c r="J64" s="6" t="inlineStr">
         <is>
           <t>el sistema no crea la cuenta e indica que las contraseñas no coinciden</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="55" customHeight="1">
-      <c r="B64" s="20" t="n"/>
-      <c r="C64" s="20" t="n"/>
-      <c r="D64" s="20" t="n"/>
-      <c r="E64" s="20" t="n"/>
-      <c r="F64" s="8" t="n">
+    <row r="65" ht="55" customHeight="1">
+      <c r="B65" s="20" t="n"/>
+      <c r="C65" s="20" t="n"/>
+      <c r="D65" s="20" t="n"/>
+      <c r="E65" s="20" t="n"/>
+      <c r="F65" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G64" s="6" t="inlineStr">
+      <c r="G65" s="6" t="inlineStr">
         <is>
           <t>Recordarme</t>
         </is>
       </c>
-      <c r="H64" s="6" t="inlineStr">
+      <c r="H65" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario inicia sesión</t>
         </is>
       </c>
-      <c r="I64" s="6" t="inlineStr">
+      <c r="I65" s="6" t="inlineStr">
         <is>
           <t>cuando marca o no marca "Recordarme"</t>
         </is>
       </c>
-      <c r="J64" s="6" t="inlineStr">
+      <c r="J65" s="6" t="inlineStr">
         <is>
           <t>si lo marcó, la sesión se mantiene hasta 30 días aunque cierre el navegador; si no, la sesión termina al cerrar el navegador</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="55" customHeight="1"/>
-    <row r="66" ht="55" customHeight="1">
-      <c r="B66" s="6" t="inlineStr">
+    <row r="66" ht="55" customHeight="1"/>
+    <row r="67" ht="55" customHeight="1">
+      <c r="B67" s="6" t="inlineStr">
         <is>
           <t>FS-HU-18</t>
         </is>
       </c>
-      <c r="C66" s="6" t="inlineStr">
+      <c r="C67" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D66" s="6" t="inlineStr">
+      <c r="D67" s="6" t="inlineStr">
         <is>
           <t>Necesito indicar mi objetivo principal y mi estilo de vida (comidas al día y horas de sueño)</t>
         </is>
       </c>
-      <c r="E66" s="6" t="inlineStr">
+      <c r="E67" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de recibir una orientación acorde a lo que busco lograr</t>
         </is>
       </c>
-      <c r="F66" s="8" t="n">
+      <c r="F67" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G66" s="6" t="inlineStr">
+      <c r="G67" s="6" t="inlineStr">
         <is>
           <t>Guardar objetivos y estilo de vida</t>
         </is>
       </c>
-      <c r="H66" s="6" t="inlineStr">
+      <c r="H67" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario completó sus datos personales en el asistente</t>
         </is>
       </c>
-      <c r="I66" s="6" t="inlineStr">
+      <c r="I67" s="6" t="inlineStr">
         <is>
           <t>cuando elige su objetivo principal, las comidas al día y las horas de sueño y presiona "Siguiente"</t>
         </is>
       </c>
-      <c r="J66" s="6" t="inlineStr">
+      <c r="J67" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda la información y avanza al paso de información de salud</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="55" customHeight="1">
-      <c r="B67" s="22" t="n"/>
-      <c r="C67" s="22" t="n"/>
-      <c r="D67" s="22" t="n"/>
-      <c r="E67" s="22" t="n"/>
-      <c r="F67" s="8" t="n">
+    <row r="68" ht="55" customHeight="1">
+      <c r="B68" s="22" t="n"/>
+      <c r="C68" s="22" t="n"/>
+      <c r="D68" s="22" t="n"/>
+      <c r="E68" s="22" t="n"/>
+      <c r="F68" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G67" s="6" t="inlineStr">
+      <c r="G68" s="6" t="inlineStr">
         <is>
           <t>Datos incompletos</t>
         </is>
       </c>
-      <c r="H67" s="6" t="inlineStr">
+      <c r="H68" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario no responde alguna de las preguntas</t>
         </is>
       </c>
-      <c r="I67" s="6" t="inlineStr">
+      <c r="I68" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Siguiente"</t>
         </is>
       </c>
-      <c r="J67" s="6" t="inlineStr">
+      <c r="J68" s="6" t="inlineStr">
         <is>
           <t>el sistema no guarda y señala cada pregunta pendiente</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="55" customHeight="1">
-      <c r="B68" s="20" t="n"/>
-      <c r="C68" s="20" t="n"/>
-      <c r="D68" s="20" t="n"/>
-      <c r="E68" s="20" t="n"/>
-      <c r="F68" s="8" t="n">
+    <row r="69" ht="55" customHeight="1">
+      <c r="B69" s="20" t="n"/>
+      <c r="C69" s="20" t="n"/>
+      <c r="D69" s="20" t="n"/>
+      <c r="E69" s="20" t="n"/>
+      <c r="F69" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G68" s="6" t="inlineStr">
+      <c r="G69" s="6" t="inlineStr">
         <is>
           <t>Editar desde el resumen</t>
         </is>
       </c>
-      <c r="H68" s="6" t="inlineStr">
+      <c r="H69" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ya completó su perfil</t>
         </is>
       </c>
-      <c r="I68" s="6" t="inlineStr">
+      <c r="I69" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Editar" en Objetivos y estilo de vida, cambia su objetivo y guarda</t>
         </is>
       </c>
-      <c r="J68" s="6" t="inlineStr">
+      <c r="J69" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda el cambio y vuelve al resumen mostrando el objetivo actualizado</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="55" customHeight="1"/>
-    <row r="70" ht="55" customHeight="1">
-      <c r="B70" s="6" t="inlineStr">
+    <row r="70" ht="55" customHeight="1"/>
+    <row r="71" ht="55" customHeight="1">
+      <c r="B71" s="6" t="inlineStr">
         <is>
           <t>FS-HU-19</t>
         </is>
       </c>
-      <c r="C70" s="6" t="inlineStr">
+      <c r="C71" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D70" s="6" t="inlineStr">
+      <c r="D71" s="6" t="inlineStr">
         <is>
           <t>Necesito registrar mis condiciones médicas, medicamentos y alergias de forma confidencial</t>
         </is>
       </c>
-      <c r="E70" s="6" t="inlineStr">
+      <c r="E71" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de recibir recomendaciones más seguras y adecuadas a mi situación</t>
         </is>
       </c>
-      <c r="F70" s="8" t="n">
+      <c r="F71" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G70" s="6" t="inlineStr">
+      <c r="G71" s="6" t="inlineStr">
         <is>
           <t>Guardar información de salud</t>
         </is>
       </c>
-      <c r="H70" s="6" t="inlineStr">
+      <c r="H71" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario está en el paso de información de salud</t>
         </is>
       </c>
-      <c r="I70" s="6" t="inlineStr">
+      <c r="I71" s="6" t="inlineStr">
         <is>
           <t>cuando marca sus condiciones médicas, indica si toma medicamentos (y de qué tipo) y sus alergias, y presiona "Siguiente"</t>
         </is>
       </c>
-      <c r="J70" s="6" t="inlineStr">
+      <c r="J71" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda la información, muestra "¡Información guardada!" con el requerimiento calórico estimado y luego el resumen del perfil</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="55" customHeight="1">
-      <c r="B71" s="22" t="n"/>
-      <c r="C71" s="22" t="n"/>
-      <c r="D71" s="22" t="n"/>
-      <c r="E71" s="22" t="n"/>
-      <c r="F71" s="8" t="n">
+    <row r="72" ht="55" customHeight="1">
+      <c r="B72" s="22" t="n"/>
+      <c r="C72" s="22" t="n"/>
+      <c r="D72" s="22" t="n"/>
+      <c r="E72" s="22" t="n"/>
+      <c r="F72" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G71" s="6" t="inlineStr">
+      <c r="G72" s="6" t="inlineStr">
         <is>
           <t>Respuestas incompletas o no válidas</t>
         </is>
       </c>
-      <c r="H71" s="6" t="inlineStr">
+      <c r="H72" s="6" t="inlineStr">
         <is>
           <t>En caso que falta una respuesta, "Ninguna" se combina con otra opción o se envía un valor fuera de la lista</t>
         </is>
       </c>
-      <c r="I71" s="6" t="inlineStr">
+      <c r="I72" s="6" t="inlineStr">
         <is>
           <t>cuando se intenta guardar</t>
         </is>
       </c>
-      <c r="J71" s="6" t="inlineStr">
+      <c r="J72" s="6" t="inlineStr">
         <is>
           <t>el sistema no guarda e indica qué respuesta corregir</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="55" customHeight="1">
-      <c r="B72" s="20" t="n"/>
-      <c r="C72" s="20" t="n"/>
-      <c r="D72" s="20" t="n"/>
-      <c r="E72" s="20" t="n"/>
-      <c r="F72" s="8" t="n">
+    <row r="73" ht="55" customHeight="1">
+      <c r="B73" s="20" t="n"/>
+      <c r="C73" s="20" t="n"/>
+      <c r="D73" s="20" t="n"/>
+      <c r="E73" s="20" t="n"/>
+      <c r="F73" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G72" s="6" t="inlineStr">
+      <c r="G73" s="6" t="inlineStr">
         <is>
           <t>Confidencialidad</t>
         </is>
       </c>
-      <c r="H72" s="6" t="inlineStr">
+      <c r="H73" s="6" t="inlineStr">
         <is>
           <t>En caso que una petición no tiene sesión válida</t>
         </is>
       </c>
-      <c r="I72" s="6" t="inlineStr">
+      <c r="I73" s="6" t="inlineStr">
         <is>
           <t>cuando intenta consultar o modificar la información de salud</t>
         </is>
       </c>
-      <c r="J72" s="6" t="inlineStr">
+      <c r="J73" s="6" t="inlineStr">
         <is>
           <t>el sistema la rechaza con código 401 sin mostrar datos</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="55" customHeight="1"/>
-    <row r="74" ht="55" customHeight="1">
-      <c r="B74" s="6" t="inlineStr">
+    <row r="74" ht="55" customHeight="1"/>
+    <row r="75" ht="55" customHeight="1">
+      <c r="B75" s="6" t="inlineStr">
         <is>
           <t>FS-HU-20</t>
         </is>
       </c>
-      <c r="C74" s="6" t="inlineStr">
+      <c r="C75" s="6" t="inlineStr">
         <is>
           <t>Como un visitante</t>
         </is>
       </c>
-      <c r="D74" s="6" t="inlineStr">
+      <c r="D75" s="6" t="inlineStr">
         <is>
           <t>Necesito conocer qué ofrece FitSearch antes de crear una cuenta o iniciar sesión</t>
         </is>
       </c>
-      <c r="E74" s="6" t="inlineStr">
+      <c r="E75" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de decidir si registrarme y acceder fácilmente a la plataforma</t>
         </is>
       </c>
-      <c r="F74" s="8" t="n">
+      <c r="F75" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G74" s="6" t="inlineStr">
+      <c r="G75" s="6" t="inlineStr">
         <is>
           <t>Ver la portada sin sesión</t>
         </is>
       </c>
-      <c r="H74" s="6" t="inlineStr">
+      <c r="H75" s="6" t="inlineStr">
         <is>
           <t>En caso que el visitante no ha iniciado sesión</t>
         </is>
       </c>
-      <c r="I74" s="6" t="inlineStr">
+      <c r="I75" s="6" t="inlineStr">
         <is>
           <t>cuando entra a FitSearch</t>
         </is>
       </c>
-      <c r="J74" s="6" t="inlineStr">
+      <c r="J75" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra la portada con lo que ofrece FitSearch (lo disponible y lo próximo) y los accesos "Iniciar sesión" y "Registrarse"</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="55" customHeight="1">
-      <c r="B75" s="22" t="n"/>
-      <c r="C75" s="22" t="n"/>
-      <c r="D75" s="22" t="n"/>
-      <c r="E75" s="22" t="n"/>
-      <c r="F75" s="8" t="n">
+    <row r="76" ht="55" customHeight="1">
+      <c r="B76" s="22" t="n"/>
+      <c r="C76" s="22" t="n"/>
+      <c r="D76" s="22" t="n"/>
+      <c r="E76" s="22" t="n"/>
+      <c r="F76" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G75" s="6" t="inlineStr">
+      <c r="G76" s="6" t="inlineStr">
         <is>
           <t>Con la sesión iniciada</t>
         </is>
       </c>
-      <c r="H75" s="6" t="inlineStr">
+      <c r="H76" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ya inició sesión</t>
         </is>
       </c>
-      <c r="I75" s="6" t="inlineStr">
+      <c r="I76" s="6" t="inlineStr">
         <is>
           <t>cuando intenta abrir la portada</t>
         </is>
       </c>
-      <c r="J75" s="6" t="inlineStr">
+      <c r="J76" s="6" t="inlineStr">
         <is>
           <t>el sistema lo lleva directamente a su Inicio</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="55" customHeight="1">
-      <c r="B76" s="20" t="n"/>
-      <c r="C76" s="20" t="n"/>
-      <c r="D76" s="20" t="n"/>
-      <c r="E76" s="20" t="n"/>
-      <c r="F76" s="8" t="n">
+    <row r="77" ht="55" customHeight="1">
+      <c r="B77" s="20" t="n"/>
+      <c r="C77" s="20" t="n"/>
+      <c r="D77" s="20" t="n"/>
+      <c r="E77" s="20" t="n"/>
+      <c r="F77" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G76" s="6" t="inlineStr">
+      <c r="G77" s="6" t="inlineStr">
         <is>
           <t>Cerrar sesión</t>
         </is>
       </c>
-      <c r="H76" s="6" t="inlineStr">
+      <c r="H77" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario tiene la sesión iniciada</t>
         </is>
       </c>
-      <c r="I76" s="6" t="inlineStr">
+      <c r="I77" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Cerrar sesión"</t>
         </is>
       </c>
-      <c r="J76" s="6" t="inlineStr">
+      <c r="J77" s="6" t="inlineStr">
         <is>
           <t>el sistema cierra la sesión y vuelve a la portada con el mensaje "Cerraste sesión correctamente"</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="55" customHeight="1"/>
-    <row r="78" ht="55" customHeight="1">
-      <c r="B78" s="6" t="inlineStr">
+    <row r="78" ht="55" customHeight="1"/>
+    <row r="79" ht="55" customHeight="1">
+      <c r="B79" s="6" t="inlineStr">
         <is>
           <t>FS-HU-21</t>
         </is>
       </c>
-      <c r="C78" s="6" t="inlineStr">
+      <c r="C79" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D78" s="6" t="inlineStr">
+      <c r="D79" s="6" t="inlineStr">
         <is>
           <t>Necesito un inicio con accesos a las secciones de la plataforma, mi objetivo, mi progreso y mis próximas citas</t>
         </is>
       </c>
-      <c r="E78" s="6" t="inlineStr">
+      <c r="E79" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de orientarme y llegar rápido a lo que necesito</t>
         </is>
       </c>
-      <c r="F78" s="8" t="n">
+      <c r="F79" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G78" s="6" t="inlineStr">
+      <c r="G79" s="6" t="inlineStr">
         <is>
           <t>Llegar al inicio</t>
         </is>
       </c>
-      <c r="H78" s="6" t="inlineStr">
+      <c r="H79" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario inicia sesión y ya eligió su tipo de cuenta</t>
         </is>
       </c>
-      <c r="I78" s="6" t="inlineStr">
+      <c r="I79" s="6" t="inlineStr">
         <is>
           <t>cuando entra a FitSearch o presiona el logo</t>
         </is>
       </c>
-      <c r="J78" s="6" t="inlineStr">
+      <c r="J79" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra el Inicio con accesos rápidos, su objetivo, su meta de calorías, sus próximas citas y profesionales destacados obtenidos de la plataforma</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="55" customHeight="1">
-      <c r="B79" s="22" t="n"/>
-      <c r="C79" s="22" t="n"/>
-      <c r="D79" s="22" t="n"/>
-      <c r="E79" s="22" t="n"/>
-      <c r="F79" s="8" t="n">
+    <row r="80" ht="55" customHeight="1">
+      <c r="B80" s="22" t="n"/>
+      <c r="C80" s="22" t="n"/>
+      <c r="D80" s="22" t="n"/>
+      <c r="E80" s="22" t="n"/>
+      <c r="F80" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G79" s="6" t="inlineStr">
+      <c r="G80" s="6" t="inlineStr">
         <is>
           <t>Sección sin datos</t>
         </is>
       </c>
-      <c r="H79" s="6" t="inlineStr">
+      <c r="H80" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario aún no define su objetivo, no tiene citas o una sección todavía no existe</t>
         </is>
       </c>
-      <c r="I79" s="6" t="inlineStr">
+      <c r="I80" s="6" t="inlineStr">
         <is>
           <t>cuando abre el Inicio o esa sección</t>
         </is>
       </c>
-      <c r="J79" s="6" t="inlineStr">
+      <c r="J80" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra un estado vacío o el aviso "Próximamente" con la acción que corresponde, sin datos inventados</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="55" customHeight="1">
-      <c r="B80" s="20" t="n"/>
-      <c r="C80" s="20" t="n"/>
-      <c r="D80" s="20" t="n"/>
-      <c r="E80" s="20" t="n"/>
-      <c r="F80" s="8" t="n">
+    <row r="81" ht="55" customHeight="1">
+      <c r="B81" s="20" t="n"/>
+      <c r="C81" s="20" t="n"/>
+      <c r="D81" s="20" t="n"/>
+      <c r="E81" s="20" t="n"/>
+      <c r="F81" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G80" s="6" t="inlineStr">
+      <c r="G81" s="6" t="inlineStr">
         <is>
           <t>Menú de la cuenta</t>
         </is>
       </c>
-      <c r="H80" s="6" t="inlineStr">
+      <c r="H81" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario tiene la sesión iniciada</t>
         </is>
       </c>
-      <c r="I80" s="6" t="inlineStr">
+      <c r="I81" s="6" t="inlineStr">
         <is>
           <t>cuando presiona "Hola, {nombre}" o su avatar</t>
         </is>
       </c>
-      <c r="J80" s="6" t="inlineStr">
+      <c r="J81" s="6" t="inlineStr">
         <is>
           <t>el sistema abre un menú con "Mi perfil" y "Cerrar sesión"; cerrar sesión vuelve a la portada</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="55" customHeight="1"/>
-    <row r="82" ht="55" customHeight="1">
-      <c r="B82" s="6" t="inlineStr">
+    <row r="82" ht="55" customHeight="1"/>
+    <row r="83" ht="55" customHeight="1">
+      <c r="B83" s="6" t="inlineStr">
         <is>
           <t>FS-HU-22</t>
         </is>
       </c>
-      <c r="C82" s="6" t="inlineStr">
+      <c r="C83" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D82" s="6" t="inlineStr">
+      <c r="D83" s="6" t="inlineStr">
         <is>
           <t>Necesito buscar profesionales por texto y filtrarlos por especialidad, comuna, distancia, calificación y modalidad</t>
         </is>
       </c>
-      <c r="E82" s="6" t="inlineStr">
+      <c r="E83" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de encontrar rápidamente al profesional que se ajusta a lo que busco</t>
         </is>
       </c>
-      <c r="F82" s="8" t="n">
+      <c r="F83" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G82" s="6" t="inlineStr">
+      <c r="G83" s="6" t="inlineStr">
         <is>
           <t>Búsqueda con filtros</t>
         </is>
       </c>
-      <c r="H82" s="6" t="inlineStr">
+      <c r="H83" s="6" t="inlineStr">
         <is>
           <t>En caso que existen profesionales registrados</t>
         </is>
       </c>
-      <c r="I82" s="6" t="inlineStr">
+      <c r="I83" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario busca un texto y elige especialidad, comuna, calificación mínima o modalidad</t>
         </is>
       </c>
-      <c r="J82" s="6" t="inlineStr">
+      <c r="J83" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra solo los profesionales que cumplen los filtros, el total encontrado y el orden elegido</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="55" customHeight="1">
-      <c r="B83" s="22" t="n"/>
-      <c r="C83" s="22" t="n"/>
-      <c r="D83" s="22" t="n"/>
-      <c r="E83" s="22" t="n"/>
-      <c r="F83" s="8" t="n">
+    <row r="84" ht="55" customHeight="1">
+      <c r="B84" s="22" t="n"/>
+      <c r="C84" s="22" t="n"/>
+      <c r="D84" s="22" t="n"/>
+      <c r="E84" s="22" t="n"/>
+      <c r="F84" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G83" s="6" t="inlineStr">
+      <c r="G84" s="6" t="inlineStr">
         <is>
           <t>Búsqueda compartida</t>
         </is>
       </c>
-      <c r="H83" s="6" t="inlineStr">
+      <c r="H84" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario copia la dirección de una búsqueda</t>
         </is>
       </c>
-      <c r="I83" s="6" t="inlineStr">
+      <c r="I84" s="6" t="inlineStr">
         <is>
           <t>cuando otra persona con sesión la abre</t>
         </is>
       </c>
-      <c r="J83" s="6" t="inlineStr">
+      <c r="J84" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra la misma búsqueda con sus filtros, porque quedan guardados en la dirección (nunca la ubicación de la persona)</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="55" customHeight="1">
-      <c r="B84" s="20" t="n"/>
-      <c r="C84" s="20" t="n"/>
-      <c r="D84" s="20" t="n"/>
-      <c r="E84" s="20" t="n"/>
-      <c r="F84" s="8" t="n">
+    <row r="85" ht="55" customHeight="1">
+      <c r="B85" s="20" t="n"/>
+      <c r="C85" s="20" t="n"/>
+      <c r="D85" s="20" t="n"/>
+      <c r="E85" s="20" t="n"/>
+      <c r="F85" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G84" s="6" t="inlineStr">
+      <c r="G85" s="6" t="inlineStr">
         <is>
           <t>Sin coincidencias</t>
         </is>
       </c>
-      <c r="H84" s="6" t="inlineStr">
+      <c r="H85" s="6" t="inlineStr">
         <is>
           <t>En caso que ningún profesional cumple los filtros</t>
         </is>
       </c>
-      <c r="I84" s="6" t="inlineStr">
+      <c r="I85" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario aplica la búsqueda</t>
         </is>
       </c>
-      <c r="J84" s="6" t="inlineStr">
+      <c r="J85" s="6" t="inlineStr">
         <is>
           <t>el sistema indica "No encontramos profesionales con esos filtros" y ofrece limpiar los filtros</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="55" customHeight="1"/>
-    <row r="86" ht="55" customHeight="1">
-      <c r="B86" s="6" t="inlineStr">
+    <row r="86" ht="55" customHeight="1"/>
+    <row r="87" ht="55" customHeight="1">
+      <c r="B87" s="6" t="inlineStr">
         <is>
           <t>FS-HU-23</t>
         </is>
       </c>
-      <c r="C86" s="6" t="inlineStr">
+      <c r="C87" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D86" s="6" t="inlineStr">
+      <c r="D87" s="6" t="inlineStr">
         <is>
           <t>Necesito guardar profesionales como favoritos</t>
         </is>
       </c>
-      <c r="E86" s="6" t="inlineStr">
+      <c r="E87" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de volver a encontrarlos fácilmente</t>
         </is>
       </c>
-      <c r="F86" s="8" t="n">
+      <c r="F87" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G86" s="6" t="inlineStr">
+      <c r="G87" s="6" t="inlineStr">
         <is>
           <t>Guardar un favorito</t>
         </is>
       </c>
-      <c r="H86" s="6" t="inlineStr">
+      <c r="H87" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ve un profesional en el Inicio, el buscador o su ficha</t>
         </is>
       </c>
-      <c r="I86" s="6" t="inlineStr">
+      <c r="I87" s="6" t="inlineStr">
         <is>
           <t>cuando presiona el corazón</t>
         </is>
       </c>
-      <c r="J86" s="6" t="inlineStr">
+      <c r="J87" s="6" t="inlineStr">
         <is>
           <t>el sistema guarda el profesional en sus favoritos y el corazón queda marcado</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="55" customHeight="1">
-      <c r="B87" s="22" t="n"/>
-      <c r="C87" s="22" t="n"/>
-      <c r="D87" s="22" t="n"/>
-      <c r="E87" s="22" t="n"/>
-      <c r="F87" s="8" t="n">
+    <row r="88" ht="55" customHeight="1">
+      <c r="B88" s="22" t="n"/>
+      <c r="C88" s="22" t="n"/>
+      <c r="D88" s="22" t="n"/>
+      <c r="E88" s="22" t="n"/>
+      <c r="F88" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G87" s="6" t="inlineStr">
+      <c r="G88" s="6" t="inlineStr">
         <is>
           <t>Ver favoritos</t>
         </is>
       </c>
-      <c r="H87" s="6" t="inlineStr">
+      <c r="H88" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario guardó profesionales</t>
         </is>
       </c>
-      <c r="I87" s="6" t="inlineStr">
+      <c r="I88" s="6" t="inlineStr">
         <is>
           <t>cuando abre "Favoritos" en el menú</t>
         </is>
       </c>
-      <c r="J87" s="6" t="inlineStr">
+      <c r="J88" s="6" t="inlineStr">
         <is>
           <t>el sistema muestra sus profesionales guardados; si no tiene ninguno, explica cómo guardarlos</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="55" customHeight="1">
-      <c r="B88" s="20" t="n"/>
-      <c r="C88" s="20" t="n"/>
-      <c r="D88" s="20" t="n"/>
-      <c r="E88" s="20" t="n"/>
-      <c r="F88" s="8" t="n">
+    <row r="89" ht="55" customHeight="1">
+      <c r="B89" s="20" t="n"/>
+      <c r="C89" s="20" t="n"/>
+      <c r="D89" s="20" t="n"/>
+      <c r="E89" s="20" t="n"/>
+      <c r="F89" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G88" s="6" t="inlineStr">
+      <c r="G89" s="6" t="inlineStr">
         <is>
           <t>Quitar un favorito</t>
         </is>
       </c>
-      <c r="H88" s="6" t="inlineStr">
+      <c r="H89" s="6" t="inlineStr">
         <is>
           <t>En caso que un profesional está en favoritos</t>
         </is>
       </c>
-      <c r="I88" s="6" t="inlineStr">
+      <c r="I89" s="6" t="inlineStr">
         <is>
           <t>cuando el usuario vuelve a presionar el corazón</t>
         </is>
       </c>
-      <c r="J88" s="6" t="inlineStr">
+      <c r="J89" s="6" t="inlineStr">
         <is>
           <t>el sistema lo quita de sus favoritos</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="55" customHeight="1"/>
-    <row r="90" ht="55" customHeight="1">
-      <c r="B90" s="6" t="inlineStr">
+    <row r="90" ht="55" customHeight="1"/>
+    <row r="91" ht="55" customHeight="1">
+      <c r="B91" s="6" t="inlineStr">
         <is>
           <t>FS-HU-24</t>
         </is>
       </c>
-      <c r="C90" s="6" t="inlineStr">
+      <c r="C91" s="6" t="inlineStr">
         <is>
           <t>Como un usuario</t>
         </is>
       </c>
-      <c r="D90" s="6" t="inlineStr">
+      <c r="D91" s="6" t="inlineStr">
         <is>
           <t>Necesito calificar con estrellas a un profesional y comentar mi experiencia</t>
         </is>
       </c>
-      <c r="E90" s="6" t="inlineStr">
+      <c r="E91" s="6" t="inlineStr">
         <is>
           <t>Con la finalidad de ayudar a otras personas a elegir y conocer la opinión de quienes ya se atendieron</t>
         </is>
       </c>
-      <c r="F90" s="8" t="n">
+      <c r="F91" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G90" s="6" t="inlineStr">
+      <c r="G91" s="6" t="inlineStr">
         <is>
           <t>Publicar una reseña</t>
         </is>
       </c>
-      <c r="H90" s="6" t="inlineStr">
+      <c r="H91" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario abre la ficha de un profesional</t>
         </is>
       </c>
-      <c r="I90" s="6" t="inlineStr">
+      <c r="I91" s="6" t="inlineStr">
         <is>
           <t>cuando elige de 1 a 5 estrellas y, si quiere, escribe un comentario de 10 a 500 caracteres</t>
         </is>
       </c>
-      <c r="J90" s="6" t="inlineStr">
+      <c r="J91" s="6" t="inlineStr">
         <is>
           <t>el sistema publica la reseña con su nombre abreviado y actualiza el promedio y la cantidad de reseñas</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="55" customHeight="1">
-      <c r="B91" s="22" t="n"/>
-      <c r="C91" s="22" t="n"/>
-      <c r="D91" s="22" t="n"/>
-      <c r="E91" s="22" t="n"/>
-      <c r="F91" s="8" t="n">
+    <row r="92" ht="55" customHeight="1">
+      <c r="B92" s="22" t="n"/>
+      <c r="C92" s="22" t="n"/>
+      <c r="D92" s="22" t="n"/>
+      <c r="E92" s="22" t="n"/>
+      <c r="F92" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G91" s="6" t="inlineStr">
+      <c r="G92" s="6" t="inlineStr">
         <is>
           <t>Editar o eliminar su reseña</t>
         </is>
       </c>
-      <c r="H91" s="6" t="inlineStr">
+      <c r="H92" s="6" t="inlineStr">
         <is>
           <t>En caso que el usuario ya calificó a ese profesional</t>
         </is>
       </c>
-      <c r="I91" s="6" t="inlineStr">
+      <c r="I92" s="6" t="inlineStr">
         <is>
           <t>cuando edita o elimina su reseña</t>
         </is>
       </c>
-      <c r="J91" s="6" t="inlineStr">
+      <c r="J92" s="6" t="inlineStr">
         <is>
           <t>el sistema reemplaza o elimina su única reseña y recalcula el promedio</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="55" customHeight="1">
-      <c r="B92" s="20" t="n"/>
-      <c r="C92" s="20" t="n"/>
-      <c r="D92" s="20" t="n"/>
-      <c r="E92" s="20" t="n"/>
-      <c r="F92" s="8" t="n">
+    <row r="93" ht="55" customHeight="1">
+      <c r="B93" s="20" t="n"/>
+      <c r="C93" s="20" t="n"/>
+      <c r="D93" s="20" t="n"/>
+      <c r="E93" s="20" t="n"/>
+      <c r="F93" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G92" s="6" t="inlineStr">
+      <c r="G93" s="6" t="inlineStr">
         <is>
           <t>Cuenta que no puede calificar</t>
         </is>
       </c>
-      <c r="H92" s="6" t="inlineStr">
+      <c r="H93" s="6" t="inlineStr">
         <is>
           <t>En caso que una cuenta profesional abre una ficha (o la suya propia)</t>
         </is>
       </c>
-      <c r="I92" s="6" t="inlineStr">
+      <c r="I93" s="6" t="inlineStr">
         <is>
           <t>cuando intenta calificar</t>
         </is>
       </c>
-      <c r="J92" s="6" t="inlineStr">
+      <c r="J93" s="6" t="inlineStr">
         <is>
           <t>el sistema le permite leer las reseñas, pero no calificar, y rechaza la calificación si se envía igual</t>
         </is>
       </c>
     </row>
-    <row r="93"/>
-    <row r="94">
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Nota:</t>
-        </is>
-      </c>
-    </row>
+    <row r="94"/>
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>- Se utilizaron 2 escenarios (criterios de aceptación) por historia de usuario: el caso principal (camino feliz) y un caso de error o borde relevante; FS-HU-14 incluye un tercer escenario para confirmar o cancelar la reserva; FS-HU-15 a FS-HU-24 también incluyen tres escenarios.</t>
+          <t>Nota:</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
+          <t>- Se utilizaron 2 escenarios (criterios de aceptación) por historia de usuario: el caso principal (camino feliz) y un caso de error o borde relevante; FS-HU-14 incluye un tercer escenario para confirmar o cancelar la reserva; FS-HU-15 a FS-HU-24 también incluyen tres escenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" t="inlineStr">
+        <is>
           <t>- El detalle completo de las 24 historias también está disponible en el Product Backlog (PMOInformatica_Plantilla_de_Product_Backlog.xlsx).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="98">
-    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="D75:D77"/>
     <mergeCell ref="G4:J4"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="B55:B57"/>
     <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D55:D57"/>
     <mergeCell ref="E26:E28"/>
     <mergeCell ref="D9:D11"/>
     <mergeCell ref="D30:D32"/>
-    <mergeCell ref="C78:C80"/>
     <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C87:C89"/>
     <mergeCell ref="D13:D14"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="D47:D48"/>
     <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E71:E73"/>
     <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="C58:C60"/>
     <mergeCell ref="B22:B24"/>
-    <mergeCell ref="E58:E60"/>
     <mergeCell ref="D22:D24"/>
-    <mergeCell ref="B62:B64"/>
-    <mergeCell ref="C43:C44"/>
-    <mergeCell ref="E82:E84"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="B70:B72"/>
-    <mergeCell ref="D70:D72"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="C63:C65"/>
+    <mergeCell ref="C59:C61"/>
+    <mergeCell ref="E59:E61"/>
+    <mergeCell ref="E50:E53"/>
     <mergeCell ref="D34:D35"/>
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="C22:C24"/>
-    <mergeCell ref="C49:C52"/>
-    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="D50:D53"/>
     <mergeCell ref="E30:E32"/>
     <mergeCell ref="E13:E14"/>
-    <mergeCell ref="E86:E88"/>
-    <mergeCell ref="D49:D52"/>
-    <mergeCell ref="B74:B76"/>
     <mergeCell ref="E22:E24"/>
-    <mergeCell ref="E62:E64"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="C62:C64"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="C54:C56"/>
+    <mergeCell ref="B83:B85"/>
+    <mergeCell ref="D83:D85"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="E63:E65"/>
     <mergeCell ref="C4:F4"/>
-    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="C79:C81"/>
+    <mergeCell ref="E79:E81"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="C26:C28"/>
-    <mergeCell ref="D86:D88"/>
     <mergeCell ref="C34:C35"/>
-    <mergeCell ref="C90:C92"/>
-    <mergeCell ref="E90:E92"/>
     <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C55:C57"/>
+    <mergeCell ref="C71:C73"/>
     <mergeCell ref="C9:C11"/>
     <mergeCell ref="E9:E11"/>
-    <mergeCell ref="E74:E76"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="D78:D80"/>
-    <mergeCell ref="D74:D76"/>
-    <mergeCell ref="C82:C84"/>
-    <mergeCell ref="D58:D60"/>
-    <mergeCell ref="C66:C68"/>
-    <mergeCell ref="E66:E68"/>
+    <mergeCell ref="C67:C69"/>
+    <mergeCell ref="B87:B89"/>
+    <mergeCell ref="D87:D89"/>
+    <mergeCell ref="D71:D73"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="E44:E45"/>
+    <mergeCell ref="D67:D69"/>
+    <mergeCell ref="E75:E77"/>
     <mergeCell ref="B26:B28"/>
     <mergeCell ref="D26:D28"/>
-    <mergeCell ref="B66:B68"/>
-    <mergeCell ref="D82:D84"/>
-    <mergeCell ref="C86:C88"/>
+    <mergeCell ref="C50:C53"/>
+    <mergeCell ref="D41:D42"/>
+    <mergeCell ref="B63:B65"/>
+    <mergeCell ref="C37:C39"/>
     <mergeCell ref="B34:B35"/>
+    <mergeCell ref="E37:E39"/>
+    <mergeCell ref="E55:E57"/>
+    <mergeCell ref="B59:B61"/>
+    <mergeCell ref="D59:D61"/>
     <mergeCell ref="C30:C32"/>
-    <mergeCell ref="D43:D44"/>
+    <mergeCell ref="B91:B93"/>
     <mergeCell ref="E16:E17"/>
-    <mergeCell ref="B49:B52"/>
-    <mergeCell ref="E78:E80"/>
-    <mergeCell ref="B86:B88"/>
+    <mergeCell ref="E87:E89"/>
+    <mergeCell ref="D91:D93"/>
     <mergeCell ref="D6:D7"/>
-    <mergeCell ref="D62:D64"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="C70:C72"/>
-    <mergeCell ref="E70:E72"/>
+    <mergeCell ref="B37:B39"/>
+    <mergeCell ref="D37:D39"/>
+    <mergeCell ref="B47:B48"/>
     <mergeCell ref="B30:B32"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="E54:E56"/>
-    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="C91:C93"/>
     <mergeCell ref="E19:E20"/>
     <mergeCell ref="E34:E35"/>
-    <mergeCell ref="B54:B56"/>
-    <mergeCell ref="D54:D56"/>
+    <mergeCell ref="D63:D65"/>
+    <mergeCell ref="E91:E93"/>
     <mergeCell ref="E6:E7"/>
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="D79:D81"/>
     <mergeCell ref="B19:B20"/>
-    <mergeCell ref="E49:E52"/>
-    <mergeCell ref="C74:C76"/>
-    <mergeCell ref="B90:B92"/>
-    <mergeCell ref="D90:D92"/>
-    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="C83:C85"/>
+    <mergeCell ref="E83:E85"/>
+    <mergeCell ref="E67:E69"/>
+    <mergeCell ref="B71:B73"/>
     <mergeCell ref="C13:C14"/>
+    <mergeCell ref="B67:B69"/>
     <mergeCell ref="D19:D20"/>
-    <mergeCell ref="B82:B84"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="C75:C77"/>
+    <mergeCell ref="E47:E48"/>
     <mergeCell ref="B9:B11"/>
-    <mergeCell ref="D66:D68"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="D44:D45"/>
   </mergeCells>
   <pageMargins left="0.7086614173228347" right="0.7086614173228347" top="0.7480314960629921" bottom="0.7480314960629921" header="0.3149606299212598" footer="0.3149606299212598"/>
   <pageSetup orientation="landscape" paperSize="9" scale="70"/>

</xml_diff>